<commit_message>
correccion de base excel
correccion de base excel
</commit_message>
<xml_diff>
--- a/evaluaciones-frontend/public/assets/formato_banco_preguntas_asig_EF_1P.xlsx
+++ b/evaluaciones-frontend/public/assets/formato_banco_preguntas_asig_EF_1P.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R65e99fdbbbd447ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banco" sheetId="3" r:id="R9465090ac55c42f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplo" sheetId="4" r:id="Ree1b56f1657e4909"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACIONES" state="veryHidden" sheetId="1" r:id="R0e1518ce15dd493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Re7d0b35c229c4d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banco" sheetId="3" r:id="Ree777055b0b24760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ejemplo" sheetId="4" r:id="R7788594530cf472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACIONES" state="veryHidden" sheetId="1" r:id="R09ff04e01f484e99"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="LISTA_TIPOS_2P">VALIDACIONES!$A$1:$A$8</x:definedName>
@@ -468,7 +468,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="66">
+  <x:fills count="76">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -568,6 +568,56 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4CCCC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4527A0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F0FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4CCCC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4527A0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F0FF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -902,7 +952,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="315">
+  <x:cellXfs count="367">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1716,6 +1766,146 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="66" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="67" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="67" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="66" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="66" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="68" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="68" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="70" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="70" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="70" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="70" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="72" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="71" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="73" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="75" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="75" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="75" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="75" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2221,10 +2411,10 @@
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="314" t="str">
+      <x:c r="A35" s="366" t="str">
         <x:v>AYUDA RÁPIDA PARA INCISOS</x:v>
       </x:c>
-      <x:c r="B35" s="314" t="str"/>
+      <x:c r="B35" s="366" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="106" t="str">
@@ -2409,40 +2599,42 @@
       <x:c r="AN1" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="AO1" s="299" t="str">
+      <x:c r="AO1" s="351" t="str">
         <x:v>CONTROL DE DISTRIBUCIÓN · 1P</x:v>
       </x:c>
-      <x:c r="AP1" s="299"/>
-      <x:c r="AQ1" s="299"/>
+      <x:c r="AP1" s="351"/>
+      <x:c r="AQ1" s="351"/>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="290"/>
-      <x:c r="B2" s="290"/>
-      <x:c r="C2" s="290"/>
-      <x:c r="D2" s="290" t="str">
+      <x:c r="A2" s="342"/>
+      <x:c r="B2" s="342"/>
+      <x:c r="C2" s="342"/>
+      <x:c r="D2" s="342" t="str">
         <x:f>IF($A2="Verdadero o Falso Simple","Verdadero",IF($A2="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A2="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E2" s="290" t="str">
+      <x:c r="E2" s="342" t="str">
         <x:f>IF($A2="Verdadero o Falso Simple","Falso",IF($A2="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A2="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F2" s="290" t="str">
+      <x:c r="F2" s="342" t="str">
         <x:f>IF($A2="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A2="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G2" s="290" t="str">
+      <x:c r="G2" s="342" t="str">
         <x:f>IF($A2="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A2="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H2" s="290" t="str">
+      <x:c r="H2" s="342" t="str">
         <x:f>IF($A2="Verdadero o Falso Simple","",IF($A2="Respuesta A/B/Ambas/Ninguna","",IF($A2="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I2" s="290"/>
-      <x:c r="J2" s="290" t="n">
+      <x:c r="I2" s="342"/>
+      <x:c r="J2" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K2" s="290" t="str">
+      <x:c r="K2" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L2" s="291"/>
-      <x:c r="M2" s="289"/>
+      <x:c r="L2" s="343" t="str">
+        <x:f>IF(TRIM($A2)="","",IF(COUNTIF($Q2:$AJ2,"?*")=0,"OK","Falta revisar: "&amp;$Q2&amp;$R2&amp;$S2&amp;$T2&amp;$U2&amp;$V2&amp;$W2&amp;$X2&amp;$Y2&amp;$Z2&amp;$AA2&amp;$AB2&amp;$AC2&amp;$AD2&amp;$AE2&amp;$AF2&amp;$AG2&amp;$AH2&amp;$AI2&amp;$AJ2))</x:f>
+      </x:c>
+      <x:c r="M2" s="341"/>
       <x:c r="N2"/>
       <x:c r="O2"/>
       <x:c r="P2"/>
@@ -2519,45 +2711,47 @@
       <x:c r="AN2" t="str">
         <x:f>IF(AND(OR($A2="Ítems agrupados por caso clínico o problema",$A2="Subítem de caso o problema",$A2="Emparejamiento Ampliado",$A2="Opción de Emparejamiento Ampliado"),TRIM($B2)=""),IF(COUNTIF($M2:$O2,"?*")&gt;0,", ","")&amp;"grupo","")</x:f>
       </x:c>
-      <x:c r="AO2" s="305" t="str">
+      <x:c r="AO2" s="357" t="str">
         <x:v>Fáciles (1)</x:v>
       </x:c>
-      <x:c r="AP2" s="306" t="n">
-        <x:f>COUNTIF($J$2:$J$61,1)</x:f>
+      <x:c r="AP2" s="358" t="n">
+        <x:f>COUNTIF($J$2:$J$1001,1)</x:f>
         <x:v>15</x:v>
       </x:c>
-      <x:c r="AQ2" s="307" t="str">
+      <x:c r="AQ2" s="359" t="str">
         <x:v>Meta: 15</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="290"/>
-      <x:c r="B3" s="290"/>
-      <x:c r="C3" s="290"/>
-      <x:c r="D3" s="290" t="str">
+      <x:c r="A3" s="342"/>
+      <x:c r="B3" s="342"/>
+      <x:c r="C3" s="342"/>
+      <x:c r="D3" s="342" t="str">
         <x:f>IF($A3="Verdadero o Falso Simple","Verdadero",IF($A3="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A3="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E3" s="290" t="str">
+      <x:c r="E3" s="342" t="str">
         <x:f>IF($A3="Verdadero o Falso Simple","Falso",IF($A3="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A3="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F3" s="290" t="str">
+      <x:c r="F3" s="342" t="str">
         <x:f>IF($A3="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A3="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G3" s="290" t="str">
+      <x:c r="G3" s="342" t="str">
         <x:f>IF($A3="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A3="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H3" s="290" t="str">
+      <x:c r="H3" s="342" t="str">
         <x:f>IF($A3="Verdadero o Falso Simple","",IF($A3="Respuesta A/B/Ambas/Ninguna","",IF($A3="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I3" s="290"/>
-      <x:c r="J3" s="290" t="n">
+      <x:c r="I3" s="342"/>
+      <x:c r="J3" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K3" s="290" t="str">
+      <x:c r="K3" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L3" s="291"/>
-      <x:c r="M3" s="289"/>
+      <x:c r="L3" s="343" t="str">
+        <x:f>IF(TRIM($A3)="","",IF(COUNTIF($Q3:$AJ3,"?*")=0,"OK","Falta revisar: "&amp;$Q3&amp;$R3&amp;$S3&amp;$T3&amp;$U3&amp;$V3&amp;$W3&amp;$X3&amp;$Y3&amp;$Z3&amp;$AA3&amp;$AB3&amp;$AC3&amp;$AD3&amp;$AE3&amp;$AF3&amp;$AG3&amp;$AH3&amp;$AI3&amp;$AJ3))</x:f>
+      </x:c>
+      <x:c r="M3" s="341"/>
       <x:c r="N3"/>
       <x:c r="O3"/>
       <x:c r="P3"/>
@@ -2634,45 +2828,47 @@
       <x:c r="AN3" t="str">
         <x:f>IF(AND(OR($A3="Ítems agrupados por caso clínico o problema",$A3="Subítem de caso o problema",$A3="Emparejamiento Ampliado",$A3="Opción de Emparejamiento Ampliado"),TRIM($B3)=""),IF(COUNTIF($M3:$O3,"?*")&gt;0,", ","")&amp;"grupo","")</x:f>
       </x:c>
-      <x:c r="AO3" s="308" t="str">
+      <x:c r="AO3" s="360" t="str">
         <x:v>Medias (2)</x:v>
       </x:c>
-      <x:c r="AP3" s="309" t="n">
-        <x:f>COUNTIF($J$2:$J$61,2)</x:f>
+      <x:c r="AP3" s="361" t="n">
+        <x:f>COUNTIF($J$2:$J$1001,2)</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="AQ3" s="310" t="str">
+      <x:c r="AQ3" s="362" t="str">
         <x:v>Meta: 30</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="290"/>
-      <x:c r="B4" s="290"/>
-      <x:c r="C4" s="290"/>
-      <x:c r="D4" s="290" t="str">
+      <x:c r="A4" s="342"/>
+      <x:c r="B4" s="342"/>
+      <x:c r="C4" s="342"/>
+      <x:c r="D4" s="342" t="str">
         <x:f>IF($A4="Verdadero o Falso Simple","Verdadero",IF($A4="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A4="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E4" s="290" t="str">
+      <x:c r="E4" s="342" t="str">
         <x:f>IF($A4="Verdadero o Falso Simple","Falso",IF($A4="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A4="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F4" s="290" t="str">
+      <x:c r="F4" s="342" t="str">
         <x:f>IF($A4="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A4="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G4" s="290" t="str">
+      <x:c r="G4" s="342" t="str">
         <x:f>IF($A4="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A4="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H4" s="290" t="str">
+      <x:c r="H4" s="342" t="str">
         <x:f>IF($A4="Verdadero o Falso Simple","",IF($A4="Respuesta A/B/Ambas/Ninguna","",IF($A4="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I4" s="290"/>
-      <x:c r="J4" s="290" t="n">
+      <x:c r="I4" s="342"/>
+      <x:c r="J4" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K4" s="290" t="str">
+      <x:c r="K4" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L4" s="291"/>
-      <x:c r="M4" s="289"/>
+      <x:c r="L4" s="343" t="str">
+        <x:f>IF(TRIM($A4)="","",IF(COUNTIF($Q4:$AJ4,"?*")=0,"OK","Falta revisar: "&amp;$Q4&amp;$R4&amp;$S4&amp;$T4&amp;$U4&amp;$V4&amp;$W4&amp;$X4&amp;$Y4&amp;$Z4&amp;$AA4&amp;$AB4&amp;$AC4&amp;$AD4&amp;$AE4&amp;$AF4&amp;$AG4&amp;$AH4&amp;$AI4&amp;$AJ4))</x:f>
+      </x:c>
+      <x:c r="M4" s="341"/>
       <x:c r="N4"/>
       <x:c r="O4"/>
       <x:c r="P4"/>
@@ -2749,45 +2945,47 @@
       <x:c r="AN4" t="str">
         <x:f>IF(AND(OR($A4="Ítems agrupados por caso clínico o problema",$A4="Subítem de caso o problema",$A4="Emparejamiento Ampliado",$A4="Opción de Emparejamiento Ampliado"),TRIM($B4)=""),IF(COUNTIF($M4:$O4,"?*")&gt;0,", ","")&amp;"grupo","")</x:f>
       </x:c>
-      <x:c r="AO4" s="308" t="str">
+      <x:c r="AO4" s="360" t="str">
         <x:v>Difíciles (3)</x:v>
       </x:c>
-      <x:c r="AP4" s="309" t="n">
-        <x:f>COUNTIF($J$2:$J$61,3)</x:f>
+      <x:c r="AP4" s="361" t="n">
+        <x:f>COUNTIF($J$2:$J$1001,3)</x:f>
         <x:v>15</x:v>
       </x:c>
-      <x:c r="AQ4" s="310" t="str">
+      <x:c r="AQ4" s="362" t="str">
         <x:v>Meta: 15</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="290"/>
-      <x:c r="B5" s="290"/>
-      <x:c r="C5" s="290"/>
-      <x:c r="D5" s="290" t="str">
+      <x:c r="A5" s="342"/>
+      <x:c r="B5" s="342"/>
+      <x:c r="C5" s="342"/>
+      <x:c r="D5" s="342" t="str">
         <x:f>IF($A5="Verdadero o Falso Simple","Verdadero",IF($A5="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A5="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E5" s="290" t="str">
+      <x:c r="E5" s="342" t="str">
         <x:f>IF($A5="Verdadero o Falso Simple","Falso",IF($A5="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A5="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F5" s="290" t="str">
+      <x:c r="F5" s="342" t="str">
         <x:f>IF($A5="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A5="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G5" s="290" t="str">
+      <x:c r="G5" s="342" t="str">
         <x:f>IF($A5="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A5="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H5" s="290" t="str">
+      <x:c r="H5" s="342" t="str">
         <x:f>IF($A5="Verdadero o Falso Simple","",IF($A5="Respuesta A/B/Ambas/Ninguna","",IF($A5="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I5" s="290"/>
-      <x:c r="J5" s="290" t="n">
+      <x:c r="I5" s="342"/>
+      <x:c r="J5" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K5" s="290" t="str">
+      <x:c r="K5" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L5" s="291"/>
-      <x:c r="M5" s="289"/>
+      <x:c r="L5" s="343" t="str">
+        <x:f>IF(TRIM($A5)="","",IF(COUNTIF($Q5:$AJ5,"?*")=0,"OK","Falta revisar: "&amp;$Q5&amp;$R5&amp;$S5&amp;$T5&amp;$U5&amp;$V5&amp;$W5&amp;$X5&amp;$Y5&amp;$Z5&amp;$AA5&amp;$AB5&amp;$AC5&amp;$AD5&amp;$AE5&amp;$AF5&amp;$AG5&amp;$AH5&amp;$AI5&amp;$AJ5))</x:f>
+      </x:c>
+      <x:c r="M5" s="341"/>
       <x:c r="N5"/>
       <x:c r="O5"/>
       <x:c r="P5"/>
@@ -2864,45 +3062,47 @@
       <x:c r="AN5" t="str">
         <x:f>IF(AND(OR($A5="Ítems agrupados por caso clínico o problema",$A5="Subítem de caso o problema",$A5="Emparejamiento Ampliado",$A5="Opción de Emparejamiento Ampliado"),TRIM($B5)=""),IF(COUNTIF($M5:$O5,"?*")&gt;0,", ","")&amp;"grupo","")</x:f>
       </x:c>
-      <x:c r="AO5" s="308" t="str">
+      <x:c r="AO5" s="360" t="str">
         <x:v>Total de ítems</x:v>
       </x:c>
-      <x:c r="AP5" s="309" t="n">
+      <x:c r="AP5" s="361" t="n">
         <x:f>SUM(AP2:AP4)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AQ5" s="310" t="str">
+      <x:c r="AQ5" s="362" t="str">
         <x:v>Meta: 60</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="290"/>
-      <x:c r="B6" s="290"/>
-      <x:c r="C6" s="290"/>
-      <x:c r="D6" s="290" t="str">
+      <x:c r="A6" s="342"/>
+      <x:c r="B6" s="342"/>
+      <x:c r="C6" s="342"/>
+      <x:c r="D6" s="342" t="str">
         <x:f>IF($A6="Verdadero o Falso Simple","Verdadero",IF($A6="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A6="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E6" s="290" t="str">
+      <x:c r="E6" s="342" t="str">
         <x:f>IF($A6="Verdadero o Falso Simple","Falso",IF($A6="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A6="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F6" s="290" t="str">
+      <x:c r="F6" s="342" t="str">
         <x:f>IF($A6="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A6="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G6" s="290" t="str">
+      <x:c r="G6" s="342" t="str">
         <x:f>IF($A6="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A6="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H6" s="290" t="str">
+      <x:c r="H6" s="342" t="str">
         <x:f>IF($A6="Verdadero o Falso Simple","",IF($A6="Respuesta A/B/Ambas/Ninguna","",IF($A6="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I6" s="290"/>
-      <x:c r="J6" s="290" t="n">
+      <x:c r="I6" s="342"/>
+      <x:c r="J6" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K6" s="290" t="str">
+      <x:c r="K6" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L6" s="291"/>
-      <x:c r="M6" s="289"/>
+      <x:c r="L6" s="343" t="str">
+        <x:f>IF(TRIM($A6)="","",IF(COUNTIF($Q6:$AJ6,"?*")=0,"OK","Falta revisar: "&amp;$Q6&amp;$R6&amp;$S6&amp;$T6&amp;$U6&amp;$V6&amp;$W6&amp;$X6&amp;$Y6&amp;$Z6&amp;$AA6&amp;$AB6&amp;$AC6&amp;$AD6&amp;$AE6&amp;$AF6&amp;$AG6&amp;$AH6&amp;$AI6&amp;$AJ6))</x:f>
+      </x:c>
+      <x:c r="M6" s="341"/>
       <x:c r="N6"/>
       <x:c r="O6"/>
       <x:c r="P6"/>
@@ -2979,43 +3179,45 @@
       <x:c r="AN6" t="str">
         <x:f>IF(AND(OR($A6="Ítems agrupados por caso clínico o problema",$A6="Subítem de caso o problema",$A6="Emparejamiento Ampliado",$A6="Opción de Emparejamiento Ampliado"),TRIM($B6)=""),IF(COUNTIF($M6:$O6,"?*")&gt;0,", ","")&amp;"grupo","")</x:f>
       </x:c>
-      <x:c r="AO6" s="311" t="str">
+      <x:c r="AO6" s="363" t="str">
         <x:v>Estado</x:v>
       </x:c>
-      <x:c r="AP6" s="312" t="str">
+      <x:c r="AP6" s="364" t="str">
         <x:f>IF(AND(AP2=15,AP3=30,AP4=15,AP5=60),"COMPLETA","REVISAR")</x:f>
         <x:v>COMPLETA</x:v>
       </x:c>
-      <x:c r="AQ6" s="313" t="str"/>
+      <x:c r="AQ6" s="365" t="str"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="290"/>
-      <x:c r="B7" s="290"/>
-      <x:c r="C7" s="290"/>
-      <x:c r="D7" s="290" t="str">
+      <x:c r="A7" s="342"/>
+      <x:c r="B7" s="342"/>
+      <x:c r="C7" s="342"/>
+      <x:c r="D7" s="342" t="str">
         <x:f>IF($A7="Verdadero o Falso Simple","Verdadero",IF($A7="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A7="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E7" s="290" t="str">
+      <x:c r="E7" s="342" t="str">
         <x:f>IF($A7="Verdadero o Falso Simple","Falso",IF($A7="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A7="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F7" s="290" t="str">
+      <x:c r="F7" s="342" t="str">
         <x:f>IF($A7="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A7="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G7" s="290" t="str">
+      <x:c r="G7" s="342" t="str">
         <x:f>IF($A7="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A7="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H7" s="290" t="str">
+      <x:c r="H7" s="342" t="str">
         <x:f>IF($A7="Verdadero o Falso Simple","",IF($A7="Respuesta A/B/Ambas/Ninguna","",IF($A7="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I7" s="290"/>
-      <x:c r="J7" s="290" t="n">
+      <x:c r="I7" s="342"/>
+      <x:c r="J7" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K7" s="290" t="str">
+      <x:c r="K7" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L7" s="291"/>
-      <x:c r="M7" s="289"/>
+      <x:c r="L7" s="343" t="str">
+        <x:f>IF(TRIM($A7)="","",IF(COUNTIF($Q7:$AJ7,"?*")=0,"OK","Falta revisar: "&amp;$Q7&amp;$R7&amp;$S7&amp;$T7&amp;$U7&amp;$V7&amp;$W7&amp;$X7&amp;$Y7&amp;$Z7&amp;$AA7&amp;$AB7&amp;$AC7&amp;$AD7&amp;$AE7&amp;$AF7&amp;$AG7&amp;$AH7&amp;$AI7&amp;$AJ7))</x:f>
+      </x:c>
+      <x:c r="M7" s="341"/>
       <x:c r="N7"/>
       <x:c r="O7"/>
       <x:c r="P7"/>
@@ -3094,33 +3296,35 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="290"/>
-      <x:c r="B8" s="290"/>
-      <x:c r="C8" s="290"/>
-      <x:c r="D8" s="290" t="str">
+      <x:c r="A8" s="342"/>
+      <x:c r="B8" s="342"/>
+      <x:c r="C8" s="342"/>
+      <x:c r="D8" s="342" t="str">
         <x:f>IF($A8="Verdadero o Falso Simple","Verdadero",IF($A8="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A8="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E8" s="290" t="str">
+      <x:c r="E8" s="342" t="str">
         <x:f>IF($A8="Verdadero o Falso Simple","Falso",IF($A8="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A8="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F8" s="290" t="str">
+      <x:c r="F8" s="342" t="str">
         <x:f>IF($A8="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A8="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G8" s="290" t="str">
+      <x:c r="G8" s="342" t="str">
         <x:f>IF($A8="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A8="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H8" s="290" t="str">
+      <x:c r="H8" s="342" t="str">
         <x:f>IF($A8="Verdadero o Falso Simple","",IF($A8="Respuesta A/B/Ambas/Ninguna","",IF($A8="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I8" s="290"/>
-      <x:c r="J8" s="290" t="n">
+      <x:c r="I8" s="342"/>
+      <x:c r="J8" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K8" s="290" t="str">
+      <x:c r="K8" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L8" s="291"/>
-      <x:c r="M8" s="289"/>
+      <x:c r="L8" s="343" t="str">
+        <x:f>IF(TRIM($A8)="","",IF(COUNTIF($Q8:$AJ8,"?*")=0,"OK","Falta revisar: "&amp;$Q8&amp;$R8&amp;$S8&amp;$T8&amp;$U8&amp;$V8&amp;$W8&amp;$X8&amp;$Y8&amp;$Z8&amp;$AA8&amp;$AB8&amp;$AC8&amp;$AD8&amp;$AE8&amp;$AF8&amp;$AG8&amp;$AH8&amp;$AI8&amp;$AJ8))</x:f>
+      </x:c>
+      <x:c r="M8" s="341"/>
       <x:c r="N8"/>
       <x:c r="O8"/>
       <x:c r="P8"/>
@@ -3199,33 +3403,35 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="290"/>
-      <x:c r="B9" s="290"/>
-      <x:c r="C9" s="290"/>
-      <x:c r="D9" s="290" t="str">
+      <x:c r="A9" s="342"/>
+      <x:c r="B9" s="342"/>
+      <x:c r="C9" s="342"/>
+      <x:c r="D9" s="342" t="str">
         <x:f>IF($A9="Verdadero o Falso Simple","Verdadero",IF($A9="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A9="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E9" s="290" t="str">
+      <x:c r="E9" s="342" t="str">
         <x:f>IF($A9="Verdadero o Falso Simple","Falso",IF($A9="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A9="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F9" s="290" t="str">
+      <x:c r="F9" s="342" t="str">
         <x:f>IF($A9="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A9="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G9" s="290" t="str">
+      <x:c r="G9" s="342" t="str">
         <x:f>IF($A9="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A9="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H9" s="290" t="str">
+      <x:c r="H9" s="342" t="str">
         <x:f>IF($A9="Verdadero o Falso Simple","",IF($A9="Respuesta A/B/Ambas/Ninguna","",IF($A9="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I9" s="290"/>
-      <x:c r="J9" s="290" t="n">
+      <x:c r="I9" s="342"/>
+      <x:c r="J9" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K9" s="290" t="str">
+      <x:c r="K9" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L9" s="291"/>
-      <x:c r="M9" s="289"/>
+      <x:c r="L9" s="343" t="str">
+        <x:f>IF(TRIM($A9)="","",IF(COUNTIF($Q9:$AJ9,"?*")=0,"OK","Falta revisar: "&amp;$Q9&amp;$R9&amp;$S9&amp;$T9&amp;$U9&amp;$V9&amp;$W9&amp;$X9&amp;$Y9&amp;$Z9&amp;$AA9&amp;$AB9&amp;$AC9&amp;$AD9&amp;$AE9&amp;$AF9&amp;$AG9&amp;$AH9&amp;$AI9&amp;$AJ9))</x:f>
+      </x:c>
+      <x:c r="M9" s="341"/>
       <x:c r="N9"/>
       <x:c r="O9"/>
       <x:c r="P9"/>
@@ -3304,33 +3510,35 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="290"/>
-      <x:c r="B10" s="290"/>
-      <x:c r="C10" s="290"/>
-      <x:c r="D10" s="290" t="str">
+      <x:c r="A10" s="342"/>
+      <x:c r="B10" s="342"/>
+      <x:c r="C10" s="342"/>
+      <x:c r="D10" s="342" t="str">
         <x:f>IF($A10="Verdadero o Falso Simple","Verdadero",IF($A10="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A10="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E10" s="290" t="str">
+      <x:c r="E10" s="342" t="str">
         <x:f>IF($A10="Verdadero o Falso Simple","Falso",IF($A10="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A10="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F10" s="290" t="str">
+      <x:c r="F10" s="342" t="str">
         <x:f>IF($A10="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A10="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G10" s="290" t="str">
+      <x:c r="G10" s="342" t="str">
         <x:f>IF($A10="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A10="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H10" s="290" t="str">
+      <x:c r="H10" s="342" t="str">
         <x:f>IF($A10="Verdadero o Falso Simple","",IF($A10="Respuesta A/B/Ambas/Ninguna","",IF($A10="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I10" s="290"/>
-      <x:c r="J10" s="290" t="n">
+      <x:c r="I10" s="342"/>
+      <x:c r="J10" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K10" s="290" t="str">
+      <x:c r="K10" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L10" s="291"/>
-      <x:c r="M10" s="289"/>
+      <x:c r="L10" s="343" t="str">
+        <x:f>IF(TRIM($A10)="","",IF(COUNTIF($Q10:$AJ10,"?*")=0,"OK","Falta revisar: "&amp;$Q10&amp;$R10&amp;$S10&amp;$T10&amp;$U10&amp;$V10&amp;$W10&amp;$X10&amp;$Y10&amp;$Z10&amp;$AA10&amp;$AB10&amp;$AC10&amp;$AD10&amp;$AE10&amp;$AF10&amp;$AG10&amp;$AH10&amp;$AI10&amp;$AJ10))</x:f>
+      </x:c>
+      <x:c r="M10" s="341"/>
       <x:c r="N10"/>
       <x:c r="O10"/>
       <x:c r="P10"/>
@@ -3409,33 +3617,35 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="290"/>
-      <x:c r="B11" s="290"/>
-      <x:c r="C11" s="290"/>
-      <x:c r="D11" s="290" t="str">
+      <x:c r="A11" s="342"/>
+      <x:c r="B11" s="342"/>
+      <x:c r="C11" s="342"/>
+      <x:c r="D11" s="342" t="str">
         <x:f>IF($A11="Verdadero o Falso Simple","Verdadero",IF($A11="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A11="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E11" s="290" t="str">
+      <x:c r="E11" s="342" t="str">
         <x:f>IF($A11="Verdadero o Falso Simple","Falso",IF($A11="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A11="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F11" s="290" t="str">
+      <x:c r="F11" s="342" t="str">
         <x:f>IF($A11="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A11="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G11" s="290" t="str">
+      <x:c r="G11" s="342" t="str">
         <x:f>IF($A11="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A11="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H11" s="290" t="str">
+      <x:c r="H11" s="342" t="str">
         <x:f>IF($A11="Verdadero o Falso Simple","",IF($A11="Respuesta A/B/Ambas/Ninguna","",IF($A11="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I11" s="290"/>
-      <x:c r="J11" s="290" t="n">
+      <x:c r="I11" s="342"/>
+      <x:c r="J11" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K11" s="290" t="str">
+      <x:c r="K11" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L11" s="291"/>
-      <x:c r="M11" s="289"/>
+      <x:c r="L11" s="343" t="str">
+        <x:f>IF(TRIM($A11)="","",IF(COUNTIF($Q11:$AJ11,"?*")=0,"OK","Falta revisar: "&amp;$Q11&amp;$R11&amp;$S11&amp;$T11&amp;$U11&amp;$V11&amp;$W11&amp;$X11&amp;$Y11&amp;$Z11&amp;$AA11&amp;$AB11&amp;$AC11&amp;$AD11&amp;$AE11&amp;$AF11&amp;$AG11&amp;$AH11&amp;$AI11&amp;$AJ11))</x:f>
+      </x:c>
+      <x:c r="M11" s="341"/>
       <x:c r="N11"/>
       <x:c r="O11"/>
       <x:c r="P11"/>
@@ -3514,33 +3724,35 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="290"/>
-      <x:c r="B12" s="290"/>
-      <x:c r="C12" s="290"/>
-      <x:c r="D12" s="290" t="str">
+      <x:c r="A12" s="342"/>
+      <x:c r="B12" s="342"/>
+      <x:c r="C12" s="342"/>
+      <x:c r="D12" s="342" t="str">
         <x:f>IF($A12="Verdadero o Falso Simple","Verdadero",IF($A12="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A12="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E12" s="290" t="str">
+      <x:c r="E12" s="342" t="str">
         <x:f>IF($A12="Verdadero o Falso Simple","Falso",IF($A12="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A12="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F12" s="290" t="str">
+      <x:c r="F12" s="342" t="str">
         <x:f>IF($A12="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A12="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G12" s="290" t="str">
+      <x:c r="G12" s="342" t="str">
         <x:f>IF($A12="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A12="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H12" s="290" t="str">
+      <x:c r="H12" s="342" t="str">
         <x:f>IF($A12="Verdadero o Falso Simple","",IF($A12="Respuesta A/B/Ambas/Ninguna","",IF($A12="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I12" s="290"/>
-      <x:c r="J12" s="290" t="n">
+      <x:c r="I12" s="342"/>
+      <x:c r="J12" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K12" s="290" t="str">
+      <x:c r="K12" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L12" s="291"/>
-      <x:c r="M12" s="289"/>
+      <x:c r="L12" s="343" t="str">
+        <x:f>IF(TRIM($A12)="","",IF(COUNTIF($Q12:$AJ12,"?*")=0,"OK","Falta revisar: "&amp;$Q12&amp;$R12&amp;$S12&amp;$T12&amp;$U12&amp;$V12&amp;$W12&amp;$X12&amp;$Y12&amp;$Z12&amp;$AA12&amp;$AB12&amp;$AC12&amp;$AD12&amp;$AE12&amp;$AF12&amp;$AG12&amp;$AH12&amp;$AI12&amp;$AJ12))</x:f>
+      </x:c>
+      <x:c r="M12" s="341"/>
       <x:c r="N12"/>
       <x:c r="O12"/>
       <x:c r="P12"/>
@@ -3619,33 +3831,35 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="290"/>
-      <x:c r="B13" s="290"/>
-      <x:c r="C13" s="290"/>
-      <x:c r="D13" s="290" t="str">
+      <x:c r="A13" s="342"/>
+      <x:c r="B13" s="342"/>
+      <x:c r="C13" s="342"/>
+      <x:c r="D13" s="342" t="str">
         <x:f>IF($A13="Verdadero o Falso Simple","Verdadero",IF($A13="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A13="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E13" s="290" t="str">
+      <x:c r="E13" s="342" t="str">
         <x:f>IF($A13="Verdadero o Falso Simple","Falso",IF($A13="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A13="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F13" s="290" t="str">
+      <x:c r="F13" s="342" t="str">
         <x:f>IF($A13="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A13="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G13" s="290" t="str">
+      <x:c r="G13" s="342" t="str">
         <x:f>IF($A13="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A13="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H13" s="290" t="str">
+      <x:c r="H13" s="342" t="str">
         <x:f>IF($A13="Verdadero o Falso Simple","",IF($A13="Respuesta A/B/Ambas/Ninguna","",IF($A13="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I13" s="290"/>
-      <x:c r="J13" s="290" t="n">
+      <x:c r="I13" s="342"/>
+      <x:c r="J13" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K13" s="290" t="str">
+      <x:c r="K13" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L13" s="291"/>
-      <x:c r="M13" s="289"/>
+      <x:c r="L13" s="343" t="str">
+        <x:f>IF(TRIM($A13)="","",IF(COUNTIF($Q13:$AJ13,"?*")=0,"OK","Falta revisar: "&amp;$Q13&amp;$R13&amp;$S13&amp;$T13&amp;$U13&amp;$V13&amp;$W13&amp;$X13&amp;$Y13&amp;$Z13&amp;$AA13&amp;$AB13&amp;$AC13&amp;$AD13&amp;$AE13&amp;$AF13&amp;$AG13&amp;$AH13&amp;$AI13&amp;$AJ13))</x:f>
+      </x:c>
+      <x:c r="M13" s="341"/>
       <x:c r="N13"/>
       <x:c r="O13"/>
       <x:c r="P13"/>
@@ -3724,33 +3938,35 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="290"/>
-      <x:c r="B14" s="290"/>
-      <x:c r="C14" s="290"/>
-      <x:c r="D14" s="290" t="str">
+      <x:c r="A14" s="342"/>
+      <x:c r="B14" s="342"/>
+      <x:c r="C14" s="342"/>
+      <x:c r="D14" s="342" t="str">
         <x:f>IF($A14="Verdadero o Falso Simple","Verdadero",IF($A14="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A14="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E14" s="290" t="str">
+      <x:c r="E14" s="342" t="str">
         <x:f>IF($A14="Verdadero o Falso Simple","Falso",IF($A14="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A14="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F14" s="290" t="str">
+      <x:c r="F14" s="342" t="str">
         <x:f>IF($A14="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A14="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G14" s="290" t="str">
+      <x:c r="G14" s="342" t="str">
         <x:f>IF($A14="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A14="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H14" s="290" t="str">
+      <x:c r="H14" s="342" t="str">
         <x:f>IF($A14="Verdadero o Falso Simple","",IF($A14="Respuesta A/B/Ambas/Ninguna","",IF($A14="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I14" s="290"/>
-      <x:c r="J14" s="290" t="n">
+      <x:c r="I14" s="342"/>
+      <x:c r="J14" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K14" s="290" t="str">
+      <x:c r="K14" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L14" s="291"/>
-      <x:c r="M14" s="289"/>
+      <x:c r="L14" s="343" t="str">
+        <x:f>IF(TRIM($A14)="","",IF(COUNTIF($Q14:$AJ14,"?*")=0,"OK","Falta revisar: "&amp;$Q14&amp;$R14&amp;$S14&amp;$T14&amp;$U14&amp;$V14&amp;$W14&amp;$X14&amp;$Y14&amp;$Z14&amp;$AA14&amp;$AB14&amp;$AC14&amp;$AD14&amp;$AE14&amp;$AF14&amp;$AG14&amp;$AH14&amp;$AI14&amp;$AJ14))</x:f>
+      </x:c>
+      <x:c r="M14" s="341"/>
       <x:c r="N14"/>
       <x:c r="O14"/>
       <x:c r="P14"/>
@@ -3829,33 +4045,35 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="290"/>
-      <x:c r="B15" s="290"/>
-      <x:c r="C15" s="290"/>
-      <x:c r="D15" s="290" t="str">
+      <x:c r="A15" s="342"/>
+      <x:c r="B15" s="342"/>
+      <x:c r="C15" s="342"/>
+      <x:c r="D15" s="342" t="str">
         <x:f>IF($A15="Verdadero o Falso Simple","Verdadero",IF($A15="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A15="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E15" s="290" t="str">
+      <x:c r="E15" s="342" t="str">
         <x:f>IF($A15="Verdadero o Falso Simple","Falso",IF($A15="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A15="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F15" s="290" t="str">
+      <x:c r="F15" s="342" t="str">
         <x:f>IF($A15="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A15="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G15" s="290" t="str">
+      <x:c r="G15" s="342" t="str">
         <x:f>IF($A15="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A15="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H15" s="290" t="str">
+      <x:c r="H15" s="342" t="str">
         <x:f>IF($A15="Verdadero o Falso Simple","",IF($A15="Respuesta A/B/Ambas/Ninguna","",IF($A15="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I15" s="290"/>
-      <x:c r="J15" s="290" t="n">
+      <x:c r="I15" s="342"/>
+      <x:c r="J15" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K15" s="290" t="str">
+      <x:c r="K15" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L15" s="291"/>
-      <x:c r="M15" s="289"/>
+      <x:c r="L15" s="343" t="str">
+        <x:f>IF(TRIM($A15)="","",IF(COUNTIF($Q15:$AJ15,"?*")=0,"OK","Falta revisar: "&amp;$Q15&amp;$R15&amp;$S15&amp;$T15&amp;$U15&amp;$V15&amp;$W15&amp;$X15&amp;$Y15&amp;$Z15&amp;$AA15&amp;$AB15&amp;$AC15&amp;$AD15&amp;$AE15&amp;$AF15&amp;$AG15&amp;$AH15&amp;$AI15&amp;$AJ15))</x:f>
+      </x:c>
+      <x:c r="M15" s="341"/>
       <x:c r="N15"/>
       <x:c r="O15"/>
       <x:c r="P15"/>
@@ -3934,33 +4152,35 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="290"/>
-      <x:c r="B16" s="290"/>
-      <x:c r="C16" s="290"/>
-      <x:c r="D16" s="290" t="str">
+      <x:c r="A16" s="342"/>
+      <x:c r="B16" s="342"/>
+      <x:c r="C16" s="342"/>
+      <x:c r="D16" s="342" t="str">
         <x:f>IF($A16="Verdadero o Falso Simple","Verdadero",IF($A16="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A16="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E16" s="290" t="str">
+      <x:c r="E16" s="342" t="str">
         <x:f>IF($A16="Verdadero o Falso Simple","Falso",IF($A16="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A16="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F16" s="290" t="str">
+      <x:c r="F16" s="342" t="str">
         <x:f>IF($A16="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A16="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G16" s="290" t="str">
+      <x:c r="G16" s="342" t="str">
         <x:f>IF($A16="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A16="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H16" s="290" t="str">
+      <x:c r="H16" s="342" t="str">
         <x:f>IF($A16="Verdadero o Falso Simple","",IF($A16="Respuesta A/B/Ambas/Ninguna","",IF($A16="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I16" s="290"/>
-      <x:c r="J16" s="290" t="n">
+      <x:c r="I16" s="342"/>
+      <x:c r="J16" s="342" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K16" s="290" t="str">
+      <x:c r="K16" s="342" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L16" s="291"/>
-      <x:c r="M16" s="289"/>
+      <x:c r="L16" s="343" t="str">
+        <x:f>IF(TRIM($A16)="","",IF(COUNTIF($Q16:$AJ16,"?*")=0,"OK","Falta revisar: "&amp;$Q16&amp;$R16&amp;$S16&amp;$T16&amp;$U16&amp;$V16&amp;$W16&amp;$X16&amp;$Y16&amp;$Z16&amp;$AA16&amp;$AB16&amp;$AC16&amp;$AD16&amp;$AE16&amp;$AF16&amp;$AG16&amp;$AH16&amp;$AI16&amp;$AJ16))</x:f>
+      </x:c>
+      <x:c r="M16" s="341"/>
       <x:c r="N16"/>
       <x:c r="O16"/>
       <x:c r="P16"/>
@@ -4039,33 +4259,35 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="292"/>
-      <x:c r="B17" s="292"/>
-      <x:c r="C17" s="292"/>
-      <x:c r="D17" s="292" t="str">
+      <x:c r="A17" s="344"/>
+      <x:c r="B17" s="344"/>
+      <x:c r="C17" s="344"/>
+      <x:c r="D17" s="344" t="str">
         <x:f>IF($A17="Verdadero o Falso Simple","Verdadero",IF($A17="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A17="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E17" s="292" t="str">
+      <x:c r="E17" s="344" t="str">
         <x:f>IF($A17="Verdadero o Falso Simple","Falso",IF($A17="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A17="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F17" s="292" t="str">
+      <x:c r="F17" s="344" t="str">
         <x:f>IF($A17="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A17="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G17" s="292" t="str">
+      <x:c r="G17" s="344" t="str">
         <x:f>IF($A17="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A17="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H17" s="292" t="str">
+      <x:c r="H17" s="344" t="str">
         <x:f>IF($A17="Verdadero o Falso Simple","",IF($A17="Respuesta A/B/Ambas/Ninguna","",IF($A17="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I17" s="292"/>
-      <x:c r="J17" s="292" t="n">
+      <x:c r="I17" s="344"/>
+      <x:c r="J17" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K17" s="292" t="str">
+      <x:c r="K17" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L17" s="293"/>
-      <x:c r="M17" s="289"/>
+      <x:c r="L17" s="345" t="str">
+        <x:f>IF(TRIM($A17)="","",IF(COUNTIF($Q17:$AJ17,"?*")=0,"OK","Falta revisar: "&amp;$Q17&amp;$R17&amp;$S17&amp;$T17&amp;$U17&amp;$V17&amp;$W17&amp;$X17&amp;$Y17&amp;$Z17&amp;$AA17&amp;$AB17&amp;$AC17&amp;$AD17&amp;$AE17&amp;$AF17&amp;$AG17&amp;$AH17&amp;$AI17&amp;$AJ17))</x:f>
+      </x:c>
+      <x:c r="M17" s="341"/>
       <x:c r="N17"/>
       <x:c r="O17"/>
       <x:c r="P17"/>
@@ -4144,33 +4366,35 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="292"/>
-      <x:c r="B18" s="292"/>
-      <x:c r="C18" s="292"/>
-      <x:c r="D18" s="292" t="str">
+      <x:c r="A18" s="344"/>
+      <x:c r="B18" s="344"/>
+      <x:c r="C18" s="344"/>
+      <x:c r="D18" s="344" t="str">
         <x:f>IF($A18="Verdadero o Falso Simple","Verdadero",IF($A18="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A18="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E18" s="292" t="str">
+      <x:c r="E18" s="344" t="str">
         <x:f>IF($A18="Verdadero o Falso Simple","Falso",IF($A18="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A18="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F18" s="292" t="str">
+      <x:c r="F18" s="344" t="str">
         <x:f>IF($A18="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A18="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G18" s="292" t="str">
+      <x:c r="G18" s="344" t="str">
         <x:f>IF($A18="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A18="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H18" s="292" t="str">
+      <x:c r="H18" s="344" t="str">
         <x:f>IF($A18="Verdadero o Falso Simple","",IF($A18="Respuesta A/B/Ambas/Ninguna","",IF($A18="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I18" s="292"/>
-      <x:c r="J18" s="292" t="n">
+      <x:c r="I18" s="344"/>
+      <x:c r="J18" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K18" s="292" t="str">
+      <x:c r="K18" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L18" s="293"/>
-      <x:c r="M18" s="289"/>
+      <x:c r="L18" s="345" t="str">
+        <x:f>IF(TRIM($A18)="","",IF(COUNTIF($Q18:$AJ18,"?*")=0,"OK","Falta revisar: "&amp;$Q18&amp;$R18&amp;$S18&amp;$T18&amp;$U18&amp;$V18&amp;$W18&amp;$X18&amp;$Y18&amp;$Z18&amp;$AA18&amp;$AB18&amp;$AC18&amp;$AD18&amp;$AE18&amp;$AF18&amp;$AG18&amp;$AH18&amp;$AI18&amp;$AJ18))</x:f>
+      </x:c>
+      <x:c r="M18" s="341"/>
       <x:c r="N18"/>
       <x:c r="O18"/>
       <x:c r="P18"/>
@@ -4249,33 +4473,35 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="292"/>
-      <x:c r="B19" s="292"/>
-      <x:c r="C19" s="292"/>
-      <x:c r="D19" s="292" t="str">
+      <x:c r="A19" s="344"/>
+      <x:c r="B19" s="344"/>
+      <x:c r="C19" s="344"/>
+      <x:c r="D19" s="344" t="str">
         <x:f>IF($A19="Verdadero o Falso Simple","Verdadero",IF($A19="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A19="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E19" s="292" t="str">
+      <x:c r="E19" s="344" t="str">
         <x:f>IF($A19="Verdadero o Falso Simple","Falso",IF($A19="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A19="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F19" s="292" t="str">
+      <x:c r="F19" s="344" t="str">
         <x:f>IF($A19="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A19="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G19" s="292" t="str">
+      <x:c r="G19" s="344" t="str">
         <x:f>IF($A19="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A19="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H19" s="292" t="str">
+      <x:c r="H19" s="344" t="str">
         <x:f>IF($A19="Verdadero o Falso Simple","",IF($A19="Respuesta A/B/Ambas/Ninguna","",IF($A19="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I19" s="292"/>
-      <x:c r="J19" s="292" t="n">
+      <x:c r="I19" s="344"/>
+      <x:c r="J19" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K19" s="292" t="str">
+      <x:c r="K19" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L19" s="293"/>
-      <x:c r="M19" s="289"/>
+      <x:c r="L19" s="345" t="str">
+        <x:f>IF(TRIM($A19)="","",IF(COUNTIF($Q19:$AJ19,"?*")=0,"OK","Falta revisar: "&amp;$Q19&amp;$R19&amp;$S19&amp;$T19&amp;$U19&amp;$V19&amp;$W19&amp;$X19&amp;$Y19&amp;$Z19&amp;$AA19&amp;$AB19&amp;$AC19&amp;$AD19&amp;$AE19&amp;$AF19&amp;$AG19&amp;$AH19&amp;$AI19&amp;$AJ19))</x:f>
+      </x:c>
+      <x:c r="M19" s="341"/>
       <x:c r="N19"/>
       <x:c r="O19"/>
       <x:c r="P19"/>
@@ -4354,33 +4580,35 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
-      <x:c r="A20" s="292"/>
-      <x:c r="B20" s="292"/>
-      <x:c r="C20" s="292"/>
-      <x:c r="D20" s="292" t="str">
+      <x:c r="A20" s="344"/>
+      <x:c r="B20" s="344"/>
+      <x:c r="C20" s="344"/>
+      <x:c r="D20" s="344" t="str">
         <x:f>IF($A20="Verdadero o Falso Simple","Verdadero",IF($A20="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A20="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E20" s="292" t="str">
+      <x:c r="E20" s="344" t="str">
         <x:f>IF($A20="Verdadero o Falso Simple","Falso",IF($A20="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A20="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F20" s="292" t="str">
+      <x:c r="F20" s="344" t="str">
         <x:f>IF($A20="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A20="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G20" s="292" t="str">
+      <x:c r="G20" s="344" t="str">
         <x:f>IF($A20="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A20="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H20" s="292" t="str">
+      <x:c r="H20" s="344" t="str">
         <x:f>IF($A20="Verdadero o Falso Simple","",IF($A20="Respuesta A/B/Ambas/Ninguna","",IF($A20="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I20" s="292"/>
-      <x:c r="J20" s="292" t="n">
+      <x:c r="I20" s="344"/>
+      <x:c r="J20" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K20" s="292" t="str">
+      <x:c r="K20" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L20" s="293"/>
-      <x:c r="M20" s="289"/>
+      <x:c r="L20" s="345" t="str">
+        <x:f>IF(TRIM($A20)="","",IF(COUNTIF($Q20:$AJ20,"?*")=0,"OK","Falta revisar: "&amp;$Q20&amp;$R20&amp;$S20&amp;$T20&amp;$U20&amp;$V20&amp;$W20&amp;$X20&amp;$Y20&amp;$Z20&amp;$AA20&amp;$AB20&amp;$AC20&amp;$AD20&amp;$AE20&amp;$AF20&amp;$AG20&amp;$AH20&amp;$AI20&amp;$AJ20))</x:f>
+      </x:c>
+      <x:c r="M20" s="341"/>
       <x:c r="N20"/>
       <x:c r="O20"/>
       <x:c r="P20"/>
@@ -4459,33 +4687,35 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
-      <x:c r="A21" s="292"/>
-      <x:c r="B21" s="292"/>
-      <x:c r="C21" s="292"/>
-      <x:c r="D21" s="292" t="str">
+      <x:c r="A21" s="344"/>
+      <x:c r="B21" s="344"/>
+      <x:c r="C21" s="344"/>
+      <x:c r="D21" s="344" t="str">
         <x:f>IF($A21="Verdadero o Falso Simple","Verdadero",IF($A21="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A21="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E21" s="292" t="str">
+      <x:c r="E21" s="344" t="str">
         <x:f>IF($A21="Verdadero o Falso Simple","Falso",IF($A21="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A21="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F21" s="292" t="str">
+      <x:c r="F21" s="344" t="str">
         <x:f>IF($A21="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A21="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G21" s="292" t="str">
+      <x:c r="G21" s="344" t="str">
         <x:f>IF($A21="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A21="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H21" s="292" t="str">
+      <x:c r="H21" s="344" t="str">
         <x:f>IF($A21="Verdadero o Falso Simple","",IF($A21="Respuesta A/B/Ambas/Ninguna","",IF($A21="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I21" s="292"/>
-      <x:c r="J21" s="292" t="n">
+      <x:c r="I21" s="344"/>
+      <x:c r="J21" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K21" s="292" t="str">
+      <x:c r="K21" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L21" s="293"/>
-      <x:c r="M21" s="289"/>
+      <x:c r="L21" s="345" t="str">
+        <x:f>IF(TRIM($A21)="","",IF(COUNTIF($Q21:$AJ21,"?*")=0,"OK","Falta revisar: "&amp;$Q21&amp;$R21&amp;$S21&amp;$T21&amp;$U21&amp;$V21&amp;$W21&amp;$X21&amp;$Y21&amp;$Z21&amp;$AA21&amp;$AB21&amp;$AC21&amp;$AD21&amp;$AE21&amp;$AF21&amp;$AG21&amp;$AH21&amp;$AI21&amp;$AJ21))</x:f>
+      </x:c>
+      <x:c r="M21" s="341"/>
       <x:c r="N21"/>
       <x:c r="O21"/>
       <x:c r="P21"/>
@@ -4564,33 +4794,35 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
-      <x:c r="A22" s="292"/>
-      <x:c r="B22" s="292"/>
-      <x:c r="C22" s="292"/>
-      <x:c r="D22" s="292" t="str">
+      <x:c r="A22" s="344"/>
+      <x:c r="B22" s="344"/>
+      <x:c r="C22" s="344"/>
+      <x:c r="D22" s="344" t="str">
         <x:f>IF($A22="Verdadero o Falso Simple","Verdadero",IF($A22="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A22="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E22" s="292" t="str">
+      <x:c r="E22" s="344" t="str">
         <x:f>IF($A22="Verdadero o Falso Simple","Falso",IF($A22="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A22="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F22" s="292" t="str">
+      <x:c r="F22" s="344" t="str">
         <x:f>IF($A22="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A22="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G22" s="292" t="str">
+      <x:c r="G22" s="344" t="str">
         <x:f>IF($A22="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A22="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H22" s="292" t="str">
+      <x:c r="H22" s="344" t="str">
         <x:f>IF($A22="Verdadero o Falso Simple","",IF($A22="Respuesta A/B/Ambas/Ninguna","",IF($A22="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I22" s="292"/>
-      <x:c r="J22" s="292" t="n">
+      <x:c r="I22" s="344"/>
+      <x:c r="J22" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K22" s="292" t="str">
+      <x:c r="K22" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L22" s="293"/>
-      <x:c r="M22" s="289"/>
+      <x:c r="L22" s="345" t="str">
+        <x:f>IF(TRIM($A22)="","",IF(COUNTIF($Q22:$AJ22,"?*")=0,"OK","Falta revisar: "&amp;$Q22&amp;$R22&amp;$S22&amp;$T22&amp;$U22&amp;$V22&amp;$W22&amp;$X22&amp;$Y22&amp;$Z22&amp;$AA22&amp;$AB22&amp;$AC22&amp;$AD22&amp;$AE22&amp;$AF22&amp;$AG22&amp;$AH22&amp;$AI22&amp;$AJ22))</x:f>
+      </x:c>
+      <x:c r="M22" s="341"/>
       <x:c r="N22"/>
       <x:c r="O22"/>
       <x:c r="P22"/>
@@ -4669,33 +4901,35 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
-      <x:c r="A23" s="292"/>
-      <x:c r="B23" s="292"/>
-      <x:c r="C23" s="292"/>
-      <x:c r="D23" s="292" t="str">
+      <x:c r="A23" s="344"/>
+      <x:c r="B23" s="344"/>
+      <x:c r="C23" s="344"/>
+      <x:c r="D23" s="344" t="str">
         <x:f>IF($A23="Verdadero o Falso Simple","Verdadero",IF($A23="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A23="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E23" s="292" t="str">
+      <x:c r="E23" s="344" t="str">
         <x:f>IF($A23="Verdadero o Falso Simple","Falso",IF($A23="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A23="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F23" s="292" t="str">
+      <x:c r="F23" s="344" t="str">
         <x:f>IF($A23="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A23="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G23" s="292" t="str">
+      <x:c r="G23" s="344" t="str">
         <x:f>IF($A23="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A23="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H23" s="292" t="str">
+      <x:c r="H23" s="344" t="str">
         <x:f>IF($A23="Verdadero o Falso Simple","",IF($A23="Respuesta A/B/Ambas/Ninguna","",IF($A23="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I23" s="292"/>
-      <x:c r="J23" s="292" t="n">
+      <x:c r="I23" s="344"/>
+      <x:c r="J23" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K23" s="292" t="str">
+      <x:c r="K23" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L23" s="293"/>
-      <x:c r="M23" s="289"/>
+      <x:c r="L23" s="345" t="str">
+        <x:f>IF(TRIM($A23)="","",IF(COUNTIF($Q23:$AJ23,"?*")=0,"OK","Falta revisar: "&amp;$Q23&amp;$R23&amp;$S23&amp;$T23&amp;$U23&amp;$V23&amp;$W23&amp;$X23&amp;$Y23&amp;$Z23&amp;$AA23&amp;$AB23&amp;$AC23&amp;$AD23&amp;$AE23&amp;$AF23&amp;$AG23&amp;$AH23&amp;$AI23&amp;$AJ23))</x:f>
+      </x:c>
+      <x:c r="M23" s="341"/>
       <x:c r="N23"/>
       <x:c r="O23"/>
       <x:c r="P23"/>
@@ -4774,33 +5008,35 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
-      <x:c r="A24" s="292"/>
-      <x:c r="B24" s="292"/>
-      <x:c r="C24" s="292"/>
-      <x:c r="D24" s="292" t="str">
+      <x:c r="A24" s="344"/>
+      <x:c r="B24" s="344"/>
+      <x:c r="C24" s="344"/>
+      <x:c r="D24" s="344" t="str">
         <x:f>IF($A24="Verdadero o Falso Simple","Verdadero",IF($A24="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A24="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E24" s="292" t="str">
+      <x:c r="E24" s="344" t="str">
         <x:f>IF($A24="Verdadero o Falso Simple","Falso",IF($A24="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A24="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F24" s="292" t="str">
+      <x:c r="F24" s="344" t="str">
         <x:f>IF($A24="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A24="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G24" s="292" t="str">
+      <x:c r="G24" s="344" t="str">
         <x:f>IF($A24="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A24="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H24" s="292" t="str">
+      <x:c r="H24" s="344" t="str">
         <x:f>IF($A24="Verdadero o Falso Simple","",IF($A24="Respuesta A/B/Ambas/Ninguna","",IF($A24="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I24" s="292"/>
-      <x:c r="J24" s="292" t="n">
+      <x:c r="I24" s="344"/>
+      <x:c r="J24" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K24" s="292" t="str">
+      <x:c r="K24" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L24" s="293"/>
-      <x:c r="M24" s="289"/>
+      <x:c r="L24" s="345" t="str">
+        <x:f>IF(TRIM($A24)="","",IF(COUNTIF($Q24:$AJ24,"?*")=0,"OK","Falta revisar: "&amp;$Q24&amp;$R24&amp;$S24&amp;$T24&amp;$U24&amp;$V24&amp;$W24&amp;$X24&amp;$Y24&amp;$Z24&amp;$AA24&amp;$AB24&amp;$AC24&amp;$AD24&amp;$AE24&amp;$AF24&amp;$AG24&amp;$AH24&amp;$AI24&amp;$AJ24))</x:f>
+      </x:c>
+      <x:c r="M24" s="341"/>
       <x:c r="N24"/>
       <x:c r="O24"/>
       <x:c r="P24"/>
@@ -4879,33 +5115,35 @@
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
-      <x:c r="A25" s="292"/>
-      <x:c r="B25" s="292"/>
-      <x:c r="C25" s="292"/>
-      <x:c r="D25" s="292" t="str">
+      <x:c r="A25" s="344"/>
+      <x:c r="B25" s="344"/>
+      <x:c r="C25" s="344"/>
+      <x:c r="D25" s="344" t="str">
         <x:f>IF($A25="Verdadero o Falso Simple","Verdadero",IF($A25="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A25="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E25" s="292" t="str">
+      <x:c r="E25" s="344" t="str">
         <x:f>IF($A25="Verdadero o Falso Simple","Falso",IF($A25="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A25="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F25" s="292" t="str">
+      <x:c r="F25" s="344" t="str">
         <x:f>IF($A25="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A25="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G25" s="292" t="str">
+      <x:c r="G25" s="344" t="str">
         <x:f>IF($A25="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A25="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H25" s="292" t="str">
+      <x:c r="H25" s="344" t="str">
         <x:f>IF($A25="Verdadero o Falso Simple","",IF($A25="Respuesta A/B/Ambas/Ninguna","",IF($A25="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I25" s="292"/>
-      <x:c r="J25" s="292" t="n">
+      <x:c r="I25" s="344"/>
+      <x:c r="J25" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K25" s="292" t="str">
+      <x:c r="K25" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L25" s="293"/>
-      <x:c r="M25" s="289"/>
+      <x:c r="L25" s="345" t="str">
+        <x:f>IF(TRIM($A25)="","",IF(COUNTIF($Q25:$AJ25,"?*")=0,"OK","Falta revisar: "&amp;$Q25&amp;$R25&amp;$S25&amp;$T25&amp;$U25&amp;$V25&amp;$W25&amp;$X25&amp;$Y25&amp;$Z25&amp;$AA25&amp;$AB25&amp;$AC25&amp;$AD25&amp;$AE25&amp;$AF25&amp;$AG25&amp;$AH25&amp;$AI25&amp;$AJ25))</x:f>
+      </x:c>
+      <x:c r="M25" s="341"/>
       <x:c r="N25"/>
       <x:c r="O25"/>
       <x:c r="P25"/>
@@ -4984,33 +5222,35 @@
       </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
-      <x:c r="A26" s="292"/>
-      <x:c r="B26" s="292"/>
-      <x:c r="C26" s="292"/>
-      <x:c r="D26" s="292" t="str">
+      <x:c r="A26" s="344"/>
+      <x:c r="B26" s="344"/>
+      <x:c r="C26" s="344"/>
+      <x:c r="D26" s="344" t="str">
         <x:f>IF($A26="Verdadero o Falso Simple","Verdadero",IF($A26="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A26="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E26" s="292" t="str">
+      <x:c r="E26" s="344" t="str">
         <x:f>IF($A26="Verdadero o Falso Simple","Falso",IF($A26="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A26="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F26" s="292" t="str">
+      <x:c r="F26" s="344" t="str">
         <x:f>IF($A26="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A26="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G26" s="292" t="str">
+      <x:c r="G26" s="344" t="str">
         <x:f>IF($A26="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A26="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H26" s="292" t="str">
+      <x:c r="H26" s="344" t="str">
         <x:f>IF($A26="Verdadero o Falso Simple","",IF($A26="Respuesta A/B/Ambas/Ninguna","",IF($A26="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I26" s="292"/>
-      <x:c r="J26" s="292" t="n">
+      <x:c r="I26" s="344"/>
+      <x:c r="J26" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K26" s="292" t="str">
+      <x:c r="K26" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L26" s="293"/>
-      <x:c r="M26" s="289"/>
+      <x:c r="L26" s="345" t="str">
+        <x:f>IF(TRIM($A26)="","",IF(COUNTIF($Q26:$AJ26,"?*")=0,"OK","Falta revisar: "&amp;$Q26&amp;$R26&amp;$S26&amp;$T26&amp;$U26&amp;$V26&amp;$W26&amp;$X26&amp;$Y26&amp;$Z26&amp;$AA26&amp;$AB26&amp;$AC26&amp;$AD26&amp;$AE26&amp;$AF26&amp;$AG26&amp;$AH26&amp;$AI26&amp;$AJ26))</x:f>
+      </x:c>
+      <x:c r="M26" s="341"/>
       <x:c r="N26"/>
       <x:c r="O26"/>
       <x:c r="P26"/>
@@ -5089,33 +5329,35 @@
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
-      <x:c r="A27" s="292"/>
-      <x:c r="B27" s="292"/>
-      <x:c r="C27" s="292"/>
-      <x:c r="D27" s="292" t="str">
+      <x:c r="A27" s="344"/>
+      <x:c r="B27" s="344"/>
+      <x:c r="C27" s="344"/>
+      <x:c r="D27" s="344" t="str">
         <x:f>IF($A27="Verdadero o Falso Simple","Verdadero",IF($A27="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A27="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E27" s="292" t="str">
+      <x:c r="E27" s="344" t="str">
         <x:f>IF($A27="Verdadero o Falso Simple","Falso",IF($A27="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A27="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F27" s="292" t="str">
+      <x:c r="F27" s="344" t="str">
         <x:f>IF($A27="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A27="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G27" s="292" t="str">
+      <x:c r="G27" s="344" t="str">
         <x:f>IF($A27="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A27="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H27" s="292" t="str">
+      <x:c r="H27" s="344" t="str">
         <x:f>IF($A27="Verdadero o Falso Simple","",IF($A27="Respuesta A/B/Ambas/Ninguna","",IF($A27="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I27" s="292"/>
-      <x:c r="J27" s="292" t="n">
+      <x:c r="I27" s="344"/>
+      <x:c r="J27" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K27" s="292" t="str">
+      <x:c r="K27" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L27" s="293"/>
-      <x:c r="M27" s="289"/>
+      <x:c r="L27" s="345" t="str">
+        <x:f>IF(TRIM($A27)="","",IF(COUNTIF($Q27:$AJ27,"?*")=0,"OK","Falta revisar: "&amp;$Q27&amp;$R27&amp;$S27&amp;$T27&amp;$U27&amp;$V27&amp;$W27&amp;$X27&amp;$Y27&amp;$Z27&amp;$AA27&amp;$AB27&amp;$AC27&amp;$AD27&amp;$AE27&amp;$AF27&amp;$AG27&amp;$AH27&amp;$AI27&amp;$AJ27))</x:f>
+      </x:c>
+      <x:c r="M27" s="341"/>
       <x:c r="N27"/>
       <x:c r="O27"/>
       <x:c r="P27"/>
@@ -5194,33 +5436,35 @@
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
-      <x:c r="A28" s="292"/>
-      <x:c r="B28" s="292"/>
-      <x:c r="C28" s="292"/>
-      <x:c r="D28" s="292" t="str">
+      <x:c r="A28" s="344"/>
+      <x:c r="B28" s="344"/>
+      <x:c r="C28" s="344"/>
+      <x:c r="D28" s="344" t="str">
         <x:f>IF($A28="Verdadero o Falso Simple","Verdadero",IF($A28="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A28="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E28" s="292" t="str">
+      <x:c r="E28" s="344" t="str">
         <x:f>IF($A28="Verdadero o Falso Simple","Falso",IF($A28="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A28="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F28" s="292" t="str">
+      <x:c r="F28" s="344" t="str">
         <x:f>IF($A28="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A28="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G28" s="292" t="str">
+      <x:c r="G28" s="344" t="str">
         <x:f>IF($A28="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A28="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H28" s="292" t="str">
+      <x:c r="H28" s="344" t="str">
         <x:f>IF($A28="Verdadero o Falso Simple","",IF($A28="Respuesta A/B/Ambas/Ninguna","",IF($A28="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I28" s="292"/>
-      <x:c r="J28" s="292" t="n">
+      <x:c r="I28" s="344"/>
+      <x:c r="J28" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K28" s="292" t="str">
+      <x:c r="K28" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L28" s="293"/>
-      <x:c r="M28" s="289"/>
+      <x:c r="L28" s="345" t="str">
+        <x:f>IF(TRIM($A28)="","",IF(COUNTIF($Q28:$AJ28,"?*")=0,"OK","Falta revisar: "&amp;$Q28&amp;$R28&amp;$S28&amp;$T28&amp;$U28&amp;$V28&amp;$W28&amp;$X28&amp;$Y28&amp;$Z28&amp;$AA28&amp;$AB28&amp;$AC28&amp;$AD28&amp;$AE28&amp;$AF28&amp;$AG28&amp;$AH28&amp;$AI28&amp;$AJ28))</x:f>
+      </x:c>
+      <x:c r="M28" s="341"/>
       <x:c r="N28"/>
       <x:c r="O28"/>
       <x:c r="P28"/>
@@ -5299,33 +5543,35 @@
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
-      <x:c r="A29" s="292"/>
-      <x:c r="B29" s="292"/>
-      <x:c r="C29" s="292"/>
-      <x:c r="D29" s="292" t="str">
+      <x:c r="A29" s="344"/>
+      <x:c r="B29" s="344"/>
+      <x:c r="C29" s="344"/>
+      <x:c r="D29" s="344" t="str">
         <x:f>IF($A29="Verdadero o Falso Simple","Verdadero",IF($A29="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A29="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E29" s="292" t="str">
+      <x:c r="E29" s="344" t="str">
         <x:f>IF($A29="Verdadero o Falso Simple","Falso",IF($A29="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A29="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F29" s="292" t="str">
+      <x:c r="F29" s="344" t="str">
         <x:f>IF($A29="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A29="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G29" s="292" t="str">
+      <x:c r="G29" s="344" t="str">
         <x:f>IF($A29="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A29="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H29" s="292" t="str">
+      <x:c r="H29" s="344" t="str">
         <x:f>IF($A29="Verdadero o Falso Simple","",IF($A29="Respuesta A/B/Ambas/Ninguna","",IF($A29="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I29" s="292"/>
-      <x:c r="J29" s="292" t="n">
+      <x:c r="I29" s="344"/>
+      <x:c r="J29" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K29" s="292" t="str">
+      <x:c r="K29" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L29" s="293"/>
-      <x:c r="M29" s="289"/>
+      <x:c r="L29" s="345" t="str">
+        <x:f>IF(TRIM($A29)="","",IF(COUNTIF($Q29:$AJ29,"?*")=0,"OK","Falta revisar: "&amp;$Q29&amp;$R29&amp;$S29&amp;$T29&amp;$U29&amp;$V29&amp;$W29&amp;$X29&amp;$Y29&amp;$Z29&amp;$AA29&amp;$AB29&amp;$AC29&amp;$AD29&amp;$AE29&amp;$AF29&amp;$AG29&amp;$AH29&amp;$AI29&amp;$AJ29))</x:f>
+      </x:c>
+      <x:c r="M29" s="341"/>
       <x:c r="N29"/>
       <x:c r="O29"/>
       <x:c r="P29"/>
@@ -5404,33 +5650,35 @@
       </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
-      <x:c r="A30" s="292"/>
-      <x:c r="B30" s="292"/>
-      <x:c r="C30" s="292"/>
-      <x:c r="D30" s="292" t="str">
+      <x:c r="A30" s="344"/>
+      <x:c r="B30" s="344"/>
+      <x:c r="C30" s="344"/>
+      <x:c r="D30" s="344" t="str">
         <x:f>IF($A30="Verdadero o Falso Simple","Verdadero",IF($A30="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A30="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E30" s="292" t="str">
+      <x:c r="E30" s="344" t="str">
         <x:f>IF($A30="Verdadero o Falso Simple","Falso",IF($A30="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A30="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F30" s="292" t="str">
+      <x:c r="F30" s="344" t="str">
         <x:f>IF($A30="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A30="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G30" s="292" t="str">
+      <x:c r="G30" s="344" t="str">
         <x:f>IF($A30="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A30="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H30" s="292" t="str">
+      <x:c r="H30" s="344" t="str">
         <x:f>IF($A30="Verdadero o Falso Simple","",IF($A30="Respuesta A/B/Ambas/Ninguna","",IF($A30="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I30" s="292"/>
-      <x:c r="J30" s="292" t="n">
+      <x:c r="I30" s="344"/>
+      <x:c r="J30" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K30" s="292" t="str">
+      <x:c r="K30" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L30" s="293"/>
-      <x:c r="M30" s="289"/>
+      <x:c r="L30" s="345" t="str">
+        <x:f>IF(TRIM($A30)="","",IF(COUNTIF($Q30:$AJ30,"?*")=0,"OK","Falta revisar: "&amp;$Q30&amp;$R30&amp;$S30&amp;$T30&amp;$U30&amp;$V30&amp;$W30&amp;$X30&amp;$Y30&amp;$Z30&amp;$AA30&amp;$AB30&amp;$AC30&amp;$AD30&amp;$AE30&amp;$AF30&amp;$AG30&amp;$AH30&amp;$AI30&amp;$AJ30))</x:f>
+      </x:c>
+      <x:c r="M30" s="341"/>
       <x:c r="N30"/>
       <x:c r="O30"/>
       <x:c r="P30"/>
@@ -5509,33 +5757,35 @@
       </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
-      <x:c r="A31" s="292"/>
-      <x:c r="B31" s="292"/>
-      <x:c r="C31" s="292"/>
-      <x:c r="D31" s="292" t="str">
+      <x:c r="A31" s="344"/>
+      <x:c r="B31" s="344"/>
+      <x:c r="C31" s="344"/>
+      <x:c r="D31" s="344" t="str">
         <x:f>IF($A31="Verdadero o Falso Simple","Verdadero",IF($A31="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A31="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E31" s="292" t="str">
+      <x:c r="E31" s="344" t="str">
         <x:f>IF($A31="Verdadero o Falso Simple","Falso",IF($A31="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A31="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F31" s="292" t="str">
+      <x:c r="F31" s="344" t="str">
         <x:f>IF($A31="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A31="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G31" s="292" t="str">
+      <x:c r="G31" s="344" t="str">
         <x:f>IF($A31="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A31="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H31" s="292" t="str">
+      <x:c r="H31" s="344" t="str">
         <x:f>IF($A31="Verdadero o Falso Simple","",IF($A31="Respuesta A/B/Ambas/Ninguna","",IF($A31="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I31" s="292"/>
-      <x:c r="J31" s="292" t="n">
+      <x:c r="I31" s="344"/>
+      <x:c r="J31" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K31" s="292" t="str">
+      <x:c r="K31" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L31" s="293"/>
-      <x:c r="M31" s="289"/>
+      <x:c r="L31" s="345" t="str">
+        <x:f>IF(TRIM($A31)="","",IF(COUNTIF($Q31:$AJ31,"?*")=0,"OK","Falta revisar: "&amp;$Q31&amp;$R31&amp;$S31&amp;$T31&amp;$U31&amp;$V31&amp;$W31&amp;$X31&amp;$Y31&amp;$Z31&amp;$AA31&amp;$AB31&amp;$AC31&amp;$AD31&amp;$AE31&amp;$AF31&amp;$AG31&amp;$AH31&amp;$AI31&amp;$AJ31))</x:f>
+      </x:c>
+      <x:c r="M31" s="341"/>
       <x:c r="N31"/>
       <x:c r="O31"/>
       <x:c r="P31"/>
@@ -5614,33 +5864,35 @@
       </x:c>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
-      <x:c r="A32" s="292"/>
-      <x:c r="B32" s="292"/>
-      <x:c r="C32" s="292"/>
-      <x:c r="D32" s="292" t="str">
+      <x:c r="A32" s="344"/>
+      <x:c r="B32" s="344"/>
+      <x:c r="C32" s="344"/>
+      <x:c r="D32" s="344" t="str">
         <x:f>IF($A32="Verdadero o Falso Simple","Verdadero",IF($A32="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A32="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E32" s="292" t="str">
+      <x:c r="E32" s="344" t="str">
         <x:f>IF($A32="Verdadero o Falso Simple","Falso",IF($A32="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A32="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F32" s="292" t="str">
+      <x:c r="F32" s="344" t="str">
         <x:f>IF($A32="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A32="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G32" s="292" t="str">
+      <x:c r="G32" s="344" t="str">
         <x:f>IF($A32="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A32="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H32" s="292" t="str">
+      <x:c r="H32" s="344" t="str">
         <x:f>IF($A32="Verdadero o Falso Simple","",IF($A32="Respuesta A/B/Ambas/Ninguna","",IF($A32="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I32" s="292"/>
-      <x:c r="J32" s="292" t="n">
+      <x:c r="I32" s="344"/>
+      <x:c r="J32" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K32" s="292" t="str">
+      <x:c r="K32" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L32" s="293"/>
-      <x:c r="M32" s="289"/>
+      <x:c r="L32" s="345" t="str">
+        <x:f>IF(TRIM($A32)="","",IF(COUNTIF($Q32:$AJ32,"?*")=0,"OK","Falta revisar: "&amp;$Q32&amp;$R32&amp;$S32&amp;$T32&amp;$U32&amp;$V32&amp;$W32&amp;$X32&amp;$Y32&amp;$Z32&amp;$AA32&amp;$AB32&amp;$AC32&amp;$AD32&amp;$AE32&amp;$AF32&amp;$AG32&amp;$AH32&amp;$AI32&amp;$AJ32))</x:f>
+      </x:c>
+      <x:c r="M32" s="341"/>
       <x:c r="N32"/>
       <x:c r="O32"/>
       <x:c r="P32"/>
@@ -5719,33 +5971,35 @@
       </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
-      <x:c r="A33" s="292"/>
-      <x:c r="B33" s="292"/>
-      <x:c r="C33" s="292"/>
-      <x:c r="D33" s="292" t="str">
+      <x:c r="A33" s="344"/>
+      <x:c r="B33" s="344"/>
+      <x:c r="C33" s="344"/>
+      <x:c r="D33" s="344" t="str">
         <x:f>IF($A33="Verdadero o Falso Simple","Verdadero",IF($A33="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A33="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E33" s="292" t="str">
+      <x:c r="E33" s="344" t="str">
         <x:f>IF($A33="Verdadero o Falso Simple","Falso",IF($A33="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A33="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F33" s="292" t="str">
+      <x:c r="F33" s="344" t="str">
         <x:f>IF($A33="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A33="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G33" s="292" t="str">
+      <x:c r="G33" s="344" t="str">
         <x:f>IF($A33="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A33="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H33" s="292" t="str">
+      <x:c r="H33" s="344" t="str">
         <x:f>IF($A33="Verdadero o Falso Simple","",IF($A33="Respuesta A/B/Ambas/Ninguna","",IF($A33="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I33" s="292"/>
-      <x:c r="J33" s="292" t="n">
+      <x:c r="I33" s="344"/>
+      <x:c r="J33" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K33" s="292" t="str">
+      <x:c r="K33" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L33" s="293"/>
-      <x:c r="M33" s="289"/>
+      <x:c r="L33" s="345" t="str">
+        <x:f>IF(TRIM($A33)="","",IF(COUNTIF($Q33:$AJ33,"?*")=0,"OK","Falta revisar: "&amp;$Q33&amp;$R33&amp;$S33&amp;$T33&amp;$U33&amp;$V33&amp;$W33&amp;$X33&amp;$Y33&amp;$Z33&amp;$AA33&amp;$AB33&amp;$AC33&amp;$AD33&amp;$AE33&amp;$AF33&amp;$AG33&amp;$AH33&amp;$AI33&amp;$AJ33))</x:f>
+      </x:c>
+      <x:c r="M33" s="341"/>
       <x:c r="N33"/>
       <x:c r="O33"/>
       <x:c r="P33"/>
@@ -5824,33 +6078,35 @@
       </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
-      <x:c r="A34" s="292"/>
-      <x:c r="B34" s="292"/>
-      <x:c r="C34" s="292"/>
-      <x:c r="D34" s="292" t="str">
+      <x:c r="A34" s="344"/>
+      <x:c r="B34" s="344"/>
+      <x:c r="C34" s="344"/>
+      <x:c r="D34" s="344" t="str">
         <x:f>IF($A34="Verdadero o Falso Simple","Verdadero",IF($A34="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A34="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E34" s="292" t="str">
+      <x:c r="E34" s="344" t="str">
         <x:f>IF($A34="Verdadero o Falso Simple","Falso",IF($A34="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A34="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F34" s="292" t="str">
+      <x:c r="F34" s="344" t="str">
         <x:f>IF($A34="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A34="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G34" s="292" t="str">
+      <x:c r="G34" s="344" t="str">
         <x:f>IF($A34="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A34="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H34" s="292" t="str">
+      <x:c r="H34" s="344" t="str">
         <x:f>IF($A34="Verdadero o Falso Simple","",IF($A34="Respuesta A/B/Ambas/Ninguna","",IF($A34="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I34" s="292"/>
-      <x:c r="J34" s="292" t="n">
+      <x:c r="I34" s="344"/>
+      <x:c r="J34" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K34" s="292" t="str">
+      <x:c r="K34" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L34" s="293"/>
-      <x:c r="M34" s="289"/>
+      <x:c r="L34" s="345" t="str">
+        <x:f>IF(TRIM($A34)="","",IF(COUNTIF($Q34:$AJ34,"?*")=0,"OK","Falta revisar: "&amp;$Q34&amp;$R34&amp;$S34&amp;$T34&amp;$U34&amp;$V34&amp;$W34&amp;$X34&amp;$Y34&amp;$Z34&amp;$AA34&amp;$AB34&amp;$AC34&amp;$AD34&amp;$AE34&amp;$AF34&amp;$AG34&amp;$AH34&amp;$AI34&amp;$AJ34))</x:f>
+      </x:c>
+      <x:c r="M34" s="341"/>
       <x:c r="N34"/>
       <x:c r="O34"/>
       <x:c r="P34"/>
@@ -5929,33 +6185,35 @@
       </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
-      <x:c r="A35" s="292"/>
-      <x:c r="B35" s="292"/>
-      <x:c r="C35" s="292"/>
-      <x:c r="D35" s="292" t="str">
+      <x:c r="A35" s="344"/>
+      <x:c r="B35" s="344"/>
+      <x:c r="C35" s="344"/>
+      <x:c r="D35" s="344" t="str">
         <x:f>IF($A35="Verdadero o Falso Simple","Verdadero",IF($A35="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A35="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E35" s="292" t="str">
+      <x:c r="E35" s="344" t="str">
         <x:f>IF($A35="Verdadero o Falso Simple","Falso",IF($A35="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A35="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F35" s="292" t="str">
+      <x:c r="F35" s="344" t="str">
         <x:f>IF($A35="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A35="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G35" s="292" t="str">
+      <x:c r="G35" s="344" t="str">
         <x:f>IF($A35="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A35="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H35" s="292" t="str">
+      <x:c r="H35" s="344" t="str">
         <x:f>IF($A35="Verdadero o Falso Simple","",IF($A35="Respuesta A/B/Ambas/Ninguna","",IF($A35="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I35" s="292"/>
-      <x:c r="J35" s="292" t="n">
+      <x:c r="I35" s="344"/>
+      <x:c r="J35" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K35" s="292" t="str">
+      <x:c r="K35" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L35" s="293"/>
-      <x:c r="M35" s="289"/>
+      <x:c r="L35" s="345" t="str">
+        <x:f>IF(TRIM($A35)="","",IF(COUNTIF($Q35:$AJ35,"?*")=0,"OK","Falta revisar: "&amp;$Q35&amp;$R35&amp;$S35&amp;$T35&amp;$U35&amp;$V35&amp;$W35&amp;$X35&amp;$Y35&amp;$Z35&amp;$AA35&amp;$AB35&amp;$AC35&amp;$AD35&amp;$AE35&amp;$AF35&amp;$AG35&amp;$AH35&amp;$AI35&amp;$AJ35))</x:f>
+      </x:c>
+      <x:c r="M35" s="341"/>
       <x:c r="N35"/>
       <x:c r="O35"/>
       <x:c r="P35"/>
@@ -6034,33 +6292,35 @@
       </x:c>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
-      <x:c r="A36" s="292"/>
-      <x:c r="B36" s="292"/>
-      <x:c r="C36" s="292"/>
-      <x:c r="D36" s="292" t="str">
+      <x:c r="A36" s="344"/>
+      <x:c r="B36" s="344"/>
+      <x:c r="C36" s="344"/>
+      <x:c r="D36" s="344" t="str">
         <x:f>IF($A36="Verdadero o Falso Simple","Verdadero",IF($A36="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A36="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E36" s="292" t="str">
+      <x:c r="E36" s="344" t="str">
         <x:f>IF($A36="Verdadero o Falso Simple","Falso",IF($A36="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A36="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F36" s="292" t="str">
+      <x:c r="F36" s="344" t="str">
         <x:f>IF($A36="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A36="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G36" s="292" t="str">
+      <x:c r="G36" s="344" t="str">
         <x:f>IF($A36="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A36="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H36" s="292" t="str">
+      <x:c r="H36" s="344" t="str">
         <x:f>IF($A36="Verdadero o Falso Simple","",IF($A36="Respuesta A/B/Ambas/Ninguna","",IF($A36="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I36" s="292"/>
-      <x:c r="J36" s="292" t="n">
+      <x:c r="I36" s="344"/>
+      <x:c r="J36" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K36" s="292" t="str">
+      <x:c r="K36" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L36" s="293"/>
-      <x:c r="M36" s="289"/>
+      <x:c r="L36" s="345" t="str">
+        <x:f>IF(TRIM($A36)="","",IF(COUNTIF($Q36:$AJ36,"?*")=0,"OK","Falta revisar: "&amp;$Q36&amp;$R36&amp;$S36&amp;$T36&amp;$U36&amp;$V36&amp;$W36&amp;$X36&amp;$Y36&amp;$Z36&amp;$AA36&amp;$AB36&amp;$AC36&amp;$AD36&amp;$AE36&amp;$AF36&amp;$AG36&amp;$AH36&amp;$AI36&amp;$AJ36))</x:f>
+      </x:c>
+      <x:c r="M36" s="341"/>
       <x:c r="N36"/>
       <x:c r="O36"/>
       <x:c r="P36"/>
@@ -6139,33 +6399,35 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
-      <x:c r="A37" s="292"/>
-      <x:c r="B37" s="292"/>
-      <x:c r="C37" s="292"/>
-      <x:c r="D37" s="292" t="str">
+      <x:c r="A37" s="344"/>
+      <x:c r="B37" s="344"/>
+      <x:c r="C37" s="344"/>
+      <x:c r="D37" s="344" t="str">
         <x:f>IF($A37="Verdadero o Falso Simple","Verdadero",IF($A37="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A37="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E37" s="292" t="str">
+      <x:c r="E37" s="344" t="str">
         <x:f>IF($A37="Verdadero o Falso Simple","Falso",IF($A37="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A37="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F37" s="292" t="str">
+      <x:c r="F37" s="344" t="str">
         <x:f>IF($A37="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A37="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G37" s="292" t="str">
+      <x:c r="G37" s="344" t="str">
         <x:f>IF($A37="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A37="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H37" s="292" t="str">
+      <x:c r="H37" s="344" t="str">
         <x:f>IF($A37="Verdadero o Falso Simple","",IF($A37="Respuesta A/B/Ambas/Ninguna","",IF($A37="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I37" s="292"/>
-      <x:c r="J37" s="292" t="n">
+      <x:c r="I37" s="344"/>
+      <x:c r="J37" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K37" s="292" t="str">
+      <x:c r="K37" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L37" s="293"/>
-      <x:c r="M37" s="289"/>
+      <x:c r="L37" s="345" t="str">
+        <x:f>IF(TRIM($A37)="","",IF(COUNTIF($Q37:$AJ37,"?*")=0,"OK","Falta revisar: "&amp;$Q37&amp;$R37&amp;$S37&amp;$T37&amp;$U37&amp;$V37&amp;$W37&amp;$X37&amp;$Y37&amp;$Z37&amp;$AA37&amp;$AB37&amp;$AC37&amp;$AD37&amp;$AE37&amp;$AF37&amp;$AG37&amp;$AH37&amp;$AI37&amp;$AJ37))</x:f>
+      </x:c>
+      <x:c r="M37" s="341"/>
       <x:c r="N37"/>
       <x:c r="O37"/>
       <x:c r="P37"/>
@@ -6244,33 +6506,35 @@
       </x:c>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
-      <x:c r="A38" s="292"/>
-      <x:c r="B38" s="292"/>
-      <x:c r="C38" s="292"/>
-      <x:c r="D38" s="292" t="str">
+      <x:c r="A38" s="344"/>
+      <x:c r="B38" s="344"/>
+      <x:c r="C38" s="344"/>
+      <x:c r="D38" s="344" t="str">
         <x:f>IF($A38="Verdadero o Falso Simple","Verdadero",IF($A38="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A38="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E38" s="292" t="str">
+      <x:c r="E38" s="344" t="str">
         <x:f>IF($A38="Verdadero o Falso Simple","Falso",IF($A38="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A38="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F38" s="292" t="str">
+      <x:c r="F38" s="344" t="str">
         <x:f>IF($A38="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A38="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G38" s="292" t="str">
+      <x:c r="G38" s="344" t="str">
         <x:f>IF($A38="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A38="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H38" s="292" t="str">
+      <x:c r="H38" s="344" t="str">
         <x:f>IF($A38="Verdadero o Falso Simple","",IF($A38="Respuesta A/B/Ambas/Ninguna","",IF($A38="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I38" s="292"/>
-      <x:c r="J38" s="292" t="n">
+      <x:c r="I38" s="344"/>
+      <x:c r="J38" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K38" s="292" t="str">
+      <x:c r="K38" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L38" s="293"/>
-      <x:c r="M38" s="289"/>
+      <x:c r="L38" s="345" t="str">
+        <x:f>IF(TRIM($A38)="","",IF(COUNTIF($Q38:$AJ38,"?*")=0,"OK","Falta revisar: "&amp;$Q38&amp;$R38&amp;$S38&amp;$T38&amp;$U38&amp;$V38&amp;$W38&amp;$X38&amp;$Y38&amp;$Z38&amp;$AA38&amp;$AB38&amp;$AC38&amp;$AD38&amp;$AE38&amp;$AF38&amp;$AG38&amp;$AH38&amp;$AI38&amp;$AJ38))</x:f>
+      </x:c>
+      <x:c r="M38" s="341"/>
       <x:c r="N38"/>
       <x:c r="O38"/>
       <x:c r="P38"/>
@@ -6349,33 +6613,35 @@
       </x:c>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
-      <x:c r="A39" s="292"/>
-      <x:c r="B39" s="292"/>
-      <x:c r="C39" s="292"/>
-      <x:c r="D39" s="292" t="str">
+      <x:c r="A39" s="344"/>
+      <x:c r="B39" s="344"/>
+      <x:c r="C39" s="344"/>
+      <x:c r="D39" s="344" t="str">
         <x:f>IF($A39="Verdadero o Falso Simple","Verdadero",IF($A39="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A39="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E39" s="292" t="str">
+      <x:c r="E39" s="344" t="str">
         <x:f>IF($A39="Verdadero o Falso Simple","Falso",IF($A39="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A39="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F39" s="292" t="str">
+      <x:c r="F39" s="344" t="str">
         <x:f>IF($A39="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A39="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G39" s="292" t="str">
+      <x:c r="G39" s="344" t="str">
         <x:f>IF($A39="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A39="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H39" s="292" t="str">
+      <x:c r="H39" s="344" t="str">
         <x:f>IF($A39="Verdadero o Falso Simple","",IF($A39="Respuesta A/B/Ambas/Ninguna","",IF($A39="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I39" s="292"/>
-      <x:c r="J39" s="292" t="n">
+      <x:c r="I39" s="344"/>
+      <x:c r="J39" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K39" s="292" t="str">
+      <x:c r="K39" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L39" s="293"/>
-      <x:c r="M39" s="289"/>
+      <x:c r="L39" s="345" t="str">
+        <x:f>IF(TRIM($A39)="","",IF(COUNTIF($Q39:$AJ39,"?*")=0,"OK","Falta revisar: "&amp;$Q39&amp;$R39&amp;$S39&amp;$T39&amp;$U39&amp;$V39&amp;$W39&amp;$X39&amp;$Y39&amp;$Z39&amp;$AA39&amp;$AB39&amp;$AC39&amp;$AD39&amp;$AE39&amp;$AF39&amp;$AG39&amp;$AH39&amp;$AI39&amp;$AJ39))</x:f>
+      </x:c>
+      <x:c r="M39" s="341"/>
       <x:c r="N39"/>
       <x:c r="O39"/>
       <x:c r="P39"/>
@@ -6454,33 +6720,35 @@
       </x:c>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
-      <x:c r="A40" s="292"/>
-      <x:c r="B40" s="292"/>
-      <x:c r="C40" s="292"/>
-      <x:c r="D40" s="292" t="str">
+      <x:c r="A40" s="344"/>
+      <x:c r="B40" s="344"/>
+      <x:c r="C40" s="344"/>
+      <x:c r="D40" s="344" t="str">
         <x:f>IF($A40="Verdadero o Falso Simple","Verdadero",IF($A40="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A40="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E40" s="292" t="str">
+      <x:c r="E40" s="344" t="str">
         <x:f>IF($A40="Verdadero o Falso Simple","Falso",IF($A40="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A40="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F40" s="292" t="str">
+      <x:c r="F40" s="344" t="str">
         <x:f>IF($A40="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A40="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G40" s="292" t="str">
+      <x:c r="G40" s="344" t="str">
         <x:f>IF($A40="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A40="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H40" s="292" t="str">
+      <x:c r="H40" s="344" t="str">
         <x:f>IF($A40="Verdadero o Falso Simple","",IF($A40="Respuesta A/B/Ambas/Ninguna","",IF($A40="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I40" s="292"/>
-      <x:c r="J40" s="292" t="n">
+      <x:c r="I40" s="344"/>
+      <x:c r="J40" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K40" s="292" t="str">
+      <x:c r="K40" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L40" s="293"/>
-      <x:c r="M40" s="289"/>
+      <x:c r="L40" s="345" t="str">
+        <x:f>IF(TRIM($A40)="","",IF(COUNTIF($Q40:$AJ40,"?*")=0,"OK","Falta revisar: "&amp;$Q40&amp;$R40&amp;$S40&amp;$T40&amp;$U40&amp;$V40&amp;$W40&amp;$X40&amp;$Y40&amp;$Z40&amp;$AA40&amp;$AB40&amp;$AC40&amp;$AD40&amp;$AE40&amp;$AF40&amp;$AG40&amp;$AH40&amp;$AI40&amp;$AJ40))</x:f>
+      </x:c>
+      <x:c r="M40" s="341"/>
       <x:c r="N40"/>
       <x:c r="O40"/>
       <x:c r="P40"/>
@@ -6559,33 +6827,35 @@
       </x:c>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
-      <x:c r="A41" s="292"/>
-      <x:c r="B41" s="292"/>
-      <x:c r="C41" s="292"/>
-      <x:c r="D41" s="292" t="str">
+      <x:c r="A41" s="344"/>
+      <x:c r="B41" s="344"/>
+      <x:c r="C41" s="344"/>
+      <x:c r="D41" s="344" t="str">
         <x:f>IF($A41="Verdadero o Falso Simple","Verdadero",IF($A41="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A41="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E41" s="292" t="str">
+      <x:c r="E41" s="344" t="str">
         <x:f>IF($A41="Verdadero o Falso Simple","Falso",IF($A41="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A41="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F41" s="292" t="str">
+      <x:c r="F41" s="344" t="str">
         <x:f>IF($A41="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A41="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G41" s="292" t="str">
+      <x:c r="G41" s="344" t="str">
         <x:f>IF($A41="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A41="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H41" s="292" t="str">
+      <x:c r="H41" s="344" t="str">
         <x:f>IF($A41="Verdadero o Falso Simple","",IF($A41="Respuesta A/B/Ambas/Ninguna","",IF($A41="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I41" s="292"/>
-      <x:c r="J41" s="292" t="n">
+      <x:c r="I41" s="344"/>
+      <x:c r="J41" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K41" s="292" t="str">
+      <x:c r="K41" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L41" s="293"/>
-      <x:c r="M41" s="289"/>
+      <x:c r="L41" s="345" t="str">
+        <x:f>IF(TRIM($A41)="","",IF(COUNTIF($Q41:$AJ41,"?*")=0,"OK","Falta revisar: "&amp;$Q41&amp;$R41&amp;$S41&amp;$T41&amp;$U41&amp;$V41&amp;$W41&amp;$X41&amp;$Y41&amp;$Z41&amp;$AA41&amp;$AB41&amp;$AC41&amp;$AD41&amp;$AE41&amp;$AF41&amp;$AG41&amp;$AH41&amp;$AI41&amp;$AJ41))</x:f>
+      </x:c>
+      <x:c r="M41" s="341"/>
       <x:c r="N41"/>
       <x:c r="O41"/>
       <x:c r="P41"/>
@@ -6664,33 +6934,35 @@
       </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
-      <x:c r="A42" s="292"/>
-      <x:c r="B42" s="292"/>
-      <x:c r="C42" s="292"/>
-      <x:c r="D42" s="292" t="str">
+      <x:c r="A42" s="344"/>
+      <x:c r="B42" s="344"/>
+      <x:c r="C42" s="344"/>
+      <x:c r="D42" s="344" t="str">
         <x:f>IF($A42="Verdadero o Falso Simple","Verdadero",IF($A42="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A42="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E42" s="292" t="str">
+      <x:c r="E42" s="344" t="str">
         <x:f>IF($A42="Verdadero o Falso Simple","Falso",IF($A42="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A42="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F42" s="292" t="str">
+      <x:c r="F42" s="344" t="str">
         <x:f>IF($A42="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A42="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G42" s="292" t="str">
+      <x:c r="G42" s="344" t="str">
         <x:f>IF($A42="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A42="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H42" s="292" t="str">
+      <x:c r="H42" s="344" t="str">
         <x:f>IF($A42="Verdadero o Falso Simple","",IF($A42="Respuesta A/B/Ambas/Ninguna","",IF($A42="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I42" s="292"/>
-      <x:c r="J42" s="292" t="n">
+      <x:c r="I42" s="344"/>
+      <x:c r="J42" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K42" s="292" t="str">
+      <x:c r="K42" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L42" s="293"/>
-      <x:c r="M42" s="289"/>
+      <x:c r="L42" s="345" t="str">
+        <x:f>IF(TRIM($A42)="","",IF(COUNTIF($Q42:$AJ42,"?*")=0,"OK","Falta revisar: "&amp;$Q42&amp;$R42&amp;$S42&amp;$T42&amp;$U42&amp;$V42&amp;$W42&amp;$X42&amp;$Y42&amp;$Z42&amp;$AA42&amp;$AB42&amp;$AC42&amp;$AD42&amp;$AE42&amp;$AF42&amp;$AG42&amp;$AH42&amp;$AI42&amp;$AJ42))</x:f>
+      </x:c>
+      <x:c r="M42" s="341"/>
       <x:c r="N42"/>
       <x:c r="O42"/>
       <x:c r="P42"/>
@@ -6769,33 +7041,35 @@
       </x:c>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
-      <x:c r="A43" s="292"/>
-      <x:c r="B43" s="292"/>
-      <x:c r="C43" s="292"/>
-      <x:c r="D43" s="292" t="str">
+      <x:c r="A43" s="344"/>
+      <x:c r="B43" s="344"/>
+      <x:c r="C43" s="344"/>
+      <x:c r="D43" s="344" t="str">
         <x:f>IF($A43="Verdadero o Falso Simple","Verdadero",IF($A43="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A43="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E43" s="292" t="str">
+      <x:c r="E43" s="344" t="str">
         <x:f>IF($A43="Verdadero o Falso Simple","Falso",IF($A43="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A43="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F43" s="292" t="str">
+      <x:c r="F43" s="344" t="str">
         <x:f>IF($A43="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A43="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G43" s="292" t="str">
+      <x:c r="G43" s="344" t="str">
         <x:f>IF($A43="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A43="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H43" s="292" t="str">
+      <x:c r="H43" s="344" t="str">
         <x:f>IF($A43="Verdadero o Falso Simple","",IF($A43="Respuesta A/B/Ambas/Ninguna","",IF($A43="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I43" s="292"/>
-      <x:c r="J43" s="292" t="n">
+      <x:c r="I43" s="344"/>
+      <x:c r="J43" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K43" s="292" t="str">
+      <x:c r="K43" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L43" s="293"/>
-      <x:c r="M43" s="289"/>
+      <x:c r="L43" s="345" t="str">
+        <x:f>IF(TRIM($A43)="","",IF(COUNTIF($Q43:$AJ43,"?*")=0,"OK","Falta revisar: "&amp;$Q43&amp;$R43&amp;$S43&amp;$T43&amp;$U43&amp;$V43&amp;$W43&amp;$X43&amp;$Y43&amp;$Z43&amp;$AA43&amp;$AB43&amp;$AC43&amp;$AD43&amp;$AE43&amp;$AF43&amp;$AG43&amp;$AH43&amp;$AI43&amp;$AJ43))</x:f>
+      </x:c>
+      <x:c r="M43" s="341"/>
       <x:c r="N43"/>
       <x:c r="O43"/>
       <x:c r="P43"/>
@@ -6874,33 +7148,35 @@
       </x:c>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
-      <x:c r="A44" s="292"/>
-      <x:c r="B44" s="292"/>
-      <x:c r="C44" s="292"/>
-      <x:c r="D44" s="292" t="str">
+      <x:c r="A44" s="344"/>
+      <x:c r="B44" s="344"/>
+      <x:c r="C44" s="344"/>
+      <x:c r="D44" s="344" t="str">
         <x:f>IF($A44="Verdadero o Falso Simple","Verdadero",IF($A44="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A44="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E44" s="292" t="str">
+      <x:c r="E44" s="344" t="str">
         <x:f>IF($A44="Verdadero o Falso Simple","Falso",IF($A44="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A44="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F44" s="292" t="str">
+      <x:c r="F44" s="344" t="str">
         <x:f>IF($A44="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A44="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G44" s="292" t="str">
+      <x:c r="G44" s="344" t="str">
         <x:f>IF($A44="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A44="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H44" s="292" t="str">
+      <x:c r="H44" s="344" t="str">
         <x:f>IF($A44="Verdadero o Falso Simple","",IF($A44="Respuesta A/B/Ambas/Ninguna","",IF($A44="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I44" s="292"/>
-      <x:c r="J44" s="292" t="n">
+      <x:c r="I44" s="344"/>
+      <x:c r="J44" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K44" s="292" t="str">
+      <x:c r="K44" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L44" s="293"/>
-      <x:c r="M44" s="289"/>
+      <x:c r="L44" s="345" t="str">
+        <x:f>IF(TRIM($A44)="","",IF(COUNTIF($Q44:$AJ44,"?*")=0,"OK","Falta revisar: "&amp;$Q44&amp;$R44&amp;$S44&amp;$T44&amp;$U44&amp;$V44&amp;$W44&amp;$X44&amp;$Y44&amp;$Z44&amp;$AA44&amp;$AB44&amp;$AC44&amp;$AD44&amp;$AE44&amp;$AF44&amp;$AG44&amp;$AH44&amp;$AI44&amp;$AJ44))</x:f>
+      </x:c>
+      <x:c r="M44" s="341"/>
       <x:c r="N44"/>
       <x:c r="O44"/>
       <x:c r="P44"/>
@@ -6979,33 +7255,35 @@
       </x:c>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
-      <x:c r="A45" s="292"/>
-      <x:c r="B45" s="292"/>
-      <x:c r="C45" s="292"/>
-      <x:c r="D45" s="292" t="str">
+      <x:c r="A45" s="344"/>
+      <x:c r="B45" s="344"/>
+      <x:c r="C45" s="344"/>
+      <x:c r="D45" s="344" t="str">
         <x:f>IF($A45="Verdadero o Falso Simple","Verdadero",IF($A45="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A45="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E45" s="292" t="str">
+      <x:c r="E45" s="344" t="str">
         <x:f>IF($A45="Verdadero o Falso Simple","Falso",IF($A45="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A45="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F45" s="292" t="str">
+      <x:c r="F45" s="344" t="str">
         <x:f>IF($A45="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A45="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G45" s="292" t="str">
+      <x:c r="G45" s="344" t="str">
         <x:f>IF($A45="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A45="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H45" s="292" t="str">
+      <x:c r="H45" s="344" t="str">
         <x:f>IF($A45="Verdadero o Falso Simple","",IF($A45="Respuesta A/B/Ambas/Ninguna","",IF($A45="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I45" s="292"/>
-      <x:c r="J45" s="292" t="n">
+      <x:c r="I45" s="344"/>
+      <x:c r="J45" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K45" s="292" t="str">
+      <x:c r="K45" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L45" s="293"/>
-      <x:c r="M45" s="289"/>
+      <x:c r="L45" s="345" t="str">
+        <x:f>IF(TRIM($A45)="","",IF(COUNTIF($Q45:$AJ45,"?*")=0,"OK","Falta revisar: "&amp;$Q45&amp;$R45&amp;$S45&amp;$T45&amp;$U45&amp;$V45&amp;$W45&amp;$X45&amp;$Y45&amp;$Z45&amp;$AA45&amp;$AB45&amp;$AC45&amp;$AD45&amp;$AE45&amp;$AF45&amp;$AG45&amp;$AH45&amp;$AI45&amp;$AJ45))</x:f>
+      </x:c>
+      <x:c r="M45" s="341"/>
       <x:c r="N45"/>
       <x:c r="O45"/>
       <x:c r="P45"/>
@@ -7084,33 +7362,35 @@
       </x:c>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
-      <x:c r="A46" s="292"/>
-      <x:c r="B46" s="292"/>
-      <x:c r="C46" s="292"/>
-      <x:c r="D46" s="292" t="str">
+      <x:c r="A46" s="344"/>
+      <x:c r="B46" s="344"/>
+      <x:c r="C46" s="344"/>
+      <x:c r="D46" s="344" t="str">
         <x:f>IF($A46="Verdadero o Falso Simple","Verdadero",IF($A46="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A46="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E46" s="292" t="str">
+      <x:c r="E46" s="344" t="str">
         <x:f>IF($A46="Verdadero o Falso Simple","Falso",IF($A46="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A46="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F46" s="292" t="str">
+      <x:c r="F46" s="344" t="str">
         <x:f>IF($A46="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A46="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G46" s="292" t="str">
+      <x:c r="G46" s="344" t="str">
         <x:f>IF($A46="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A46="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H46" s="292" t="str">
+      <x:c r="H46" s="344" t="str">
         <x:f>IF($A46="Verdadero o Falso Simple","",IF($A46="Respuesta A/B/Ambas/Ninguna","",IF($A46="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I46" s="292"/>
-      <x:c r="J46" s="292" t="n">
+      <x:c r="I46" s="344"/>
+      <x:c r="J46" s="344" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K46" s="292" t="str">
+      <x:c r="K46" s="344" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L46" s="293"/>
-      <x:c r="M46" s="289"/>
+      <x:c r="L46" s="345" t="str">
+        <x:f>IF(TRIM($A46)="","",IF(COUNTIF($Q46:$AJ46,"?*")=0,"OK","Falta revisar: "&amp;$Q46&amp;$R46&amp;$S46&amp;$T46&amp;$U46&amp;$V46&amp;$W46&amp;$X46&amp;$Y46&amp;$Z46&amp;$AA46&amp;$AB46&amp;$AC46&amp;$AD46&amp;$AE46&amp;$AF46&amp;$AG46&amp;$AH46&amp;$AI46&amp;$AJ46))</x:f>
+      </x:c>
+      <x:c r="M46" s="341"/>
       <x:c r="N46"/>
       <x:c r="O46"/>
       <x:c r="P46"/>
@@ -7189,33 +7469,35 @@
       </x:c>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
-      <x:c r="A47" s="294"/>
-      <x:c r="B47" s="294"/>
-      <x:c r="C47" s="294"/>
-      <x:c r="D47" s="294" t="str">
+      <x:c r="A47" s="346"/>
+      <x:c r="B47" s="346"/>
+      <x:c r="C47" s="346"/>
+      <x:c r="D47" s="346" t="str">
         <x:f>IF($A47="Verdadero o Falso Simple","Verdadero",IF($A47="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A47="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E47" s="294" t="str">
+      <x:c r="E47" s="346" t="str">
         <x:f>IF($A47="Verdadero o Falso Simple","Falso",IF($A47="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A47="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F47" s="294" t="str">
+      <x:c r="F47" s="346" t="str">
         <x:f>IF($A47="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A47="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G47" s="294" t="str">
+      <x:c r="G47" s="346" t="str">
         <x:f>IF($A47="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A47="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H47" s="294" t="str">
+      <x:c r="H47" s="346" t="str">
         <x:f>IF($A47="Verdadero o Falso Simple","",IF($A47="Respuesta A/B/Ambas/Ninguna","",IF($A47="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I47" s="294"/>
-      <x:c r="J47" s="294" t="n">
+      <x:c r="I47" s="346"/>
+      <x:c r="J47" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K47" s="294" t="str">
+      <x:c r="K47" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L47" s="295"/>
-      <x:c r="M47" s="289"/>
+      <x:c r="L47" s="347" t="str">
+        <x:f>IF(TRIM($A47)="","",IF(COUNTIF($Q47:$AJ47,"?*")=0,"OK","Falta revisar: "&amp;$Q47&amp;$R47&amp;$S47&amp;$T47&amp;$U47&amp;$V47&amp;$W47&amp;$X47&amp;$Y47&amp;$Z47&amp;$AA47&amp;$AB47&amp;$AC47&amp;$AD47&amp;$AE47&amp;$AF47&amp;$AG47&amp;$AH47&amp;$AI47&amp;$AJ47))</x:f>
+      </x:c>
+      <x:c r="M47" s="341"/>
       <x:c r="N47"/>
       <x:c r="O47"/>
       <x:c r="P47"/>
@@ -7294,33 +7576,35 @@
       </x:c>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
-      <x:c r="A48" s="294"/>
-      <x:c r="B48" s="294"/>
-      <x:c r="C48" s="294"/>
-      <x:c r="D48" s="294" t="str">
+      <x:c r="A48" s="346"/>
+      <x:c r="B48" s="346"/>
+      <x:c r="C48" s="346"/>
+      <x:c r="D48" s="346" t="str">
         <x:f>IF($A48="Verdadero o Falso Simple","Verdadero",IF($A48="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A48="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E48" s="294" t="str">
+      <x:c r="E48" s="346" t="str">
         <x:f>IF($A48="Verdadero o Falso Simple","Falso",IF($A48="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A48="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F48" s="294" t="str">
+      <x:c r="F48" s="346" t="str">
         <x:f>IF($A48="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A48="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G48" s="294" t="str">
+      <x:c r="G48" s="346" t="str">
         <x:f>IF($A48="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A48="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H48" s="294" t="str">
+      <x:c r="H48" s="346" t="str">
         <x:f>IF($A48="Verdadero o Falso Simple","",IF($A48="Respuesta A/B/Ambas/Ninguna","",IF($A48="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I48" s="294"/>
-      <x:c r="J48" s="294" t="n">
+      <x:c r="I48" s="346"/>
+      <x:c r="J48" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K48" s="294" t="str">
+      <x:c r="K48" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L48" s="295"/>
-      <x:c r="M48" s="289"/>
+      <x:c r="L48" s="347" t="str">
+        <x:f>IF(TRIM($A48)="","",IF(COUNTIF($Q48:$AJ48,"?*")=0,"OK","Falta revisar: "&amp;$Q48&amp;$R48&amp;$S48&amp;$T48&amp;$U48&amp;$V48&amp;$W48&amp;$X48&amp;$Y48&amp;$Z48&amp;$AA48&amp;$AB48&amp;$AC48&amp;$AD48&amp;$AE48&amp;$AF48&amp;$AG48&amp;$AH48&amp;$AI48&amp;$AJ48))</x:f>
+      </x:c>
+      <x:c r="M48" s="341"/>
       <x:c r="N48"/>
       <x:c r="O48"/>
       <x:c r="P48"/>
@@ -7399,33 +7683,35 @@
       </x:c>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
-      <x:c r="A49" s="294"/>
-      <x:c r="B49" s="294"/>
-      <x:c r="C49" s="294"/>
-      <x:c r="D49" s="294" t="str">
+      <x:c r="A49" s="346"/>
+      <x:c r="B49" s="346"/>
+      <x:c r="C49" s="346"/>
+      <x:c r="D49" s="346" t="str">
         <x:f>IF($A49="Verdadero o Falso Simple","Verdadero",IF($A49="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A49="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E49" s="294" t="str">
+      <x:c r="E49" s="346" t="str">
         <x:f>IF($A49="Verdadero o Falso Simple","Falso",IF($A49="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A49="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F49" s="294" t="str">
+      <x:c r="F49" s="346" t="str">
         <x:f>IF($A49="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A49="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G49" s="294" t="str">
+      <x:c r="G49" s="346" t="str">
         <x:f>IF($A49="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A49="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H49" s="294" t="str">
+      <x:c r="H49" s="346" t="str">
         <x:f>IF($A49="Verdadero o Falso Simple","",IF($A49="Respuesta A/B/Ambas/Ninguna","",IF($A49="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I49" s="294"/>
-      <x:c r="J49" s="294" t="n">
+      <x:c r="I49" s="346"/>
+      <x:c r="J49" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K49" s="294" t="str">
+      <x:c r="K49" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L49" s="295"/>
-      <x:c r="M49" s="289"/>
+      <x:c r="L49" s="347" t="str">
+        <x:f>IF(TRIM($A49)="","",IF(COUNTIF($Q49:$AJ49,"?*")=0,"OK","Falta revisar: "&amp;$Q49&amp;$R49&amp;$S49&amp;$T49&amp;$U49&amp;$V49&amp;$W49&amp;$X49&amp;$Y49&amp;$Z49&amp;$AA49&amp;$AB49&amp;$AC49&amp;$AD49&amp;$AE49&amp;$AF49&amp;$AG49&amp;$AH49&amp;$AI49&amp;$AJ49))</x:f>
+      </x:c>
+      <x:c r="M49" s="341"/>
       <x:c r="N49"/>
       <x:c r="O49"/>
       <x:c r="P49"/>
@@ -7504,33 +7790,35 @@
       </x:c>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
-      <x:c r="A50" s="294"/>
-      <x:c r="B50" s="294"/>
-      <x:c r="C50" s="294"/>
-      <x:c r="D50" s="294" t="str">
+      <x:c r="A50" s="346"/>
+      <x:c r="B50" s="346"/>
+      <x:c r="C50" s="346"/>
+      <x:c r="D50" s="346" t="str">
         <x:f>IF($A50="Verdadero o Falso Simple","Verdadero",IF($A50="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A50="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E50" s="294" t="str">
+      <x:c r="E50" s="346" t="str">
         <x:f>IF($A50="Verdadero o Falso Simple","Falso",IF($A50="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A50="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F50" s="294" t="str">
+      <x:c r="F50" s="346" t="str">
         <x:f>IF($A50="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A50="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G50" s="294" t="str">
+      <x:c r="G50" s="346" t="str">
         <x:f>IF($A50="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A50="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H50" s="294" t="str">
+      <x:c r="H50" s="346" t="str">
         <x:f>IF($A50="Verdadero o Falso Simple","",IF($A50="Respuesta A/B/Ambas/Ninguna","",IF($A50="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I50" s="294"/>
-      <x:c r="J50" s="294" t="n">
+      <x:c r="I50" s="346"/>
+      <x:c r="J50" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K50" s="294" t="str">
+      <x:c r="K50" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L50" s="295"/>
-      <x:c r="M50" s="289"/>
+      <x:c r="L50" s="347" t="str">
+        <x:f>IF(TRIM($A50)="","",IF(COUNTIF($Q50:$AJ50,"?*")=0,"OK","Falta revisar: "&amp;$Q50&amp;$R50&amp;$S50&amp;$T50&amp;$U50&amp;$V50&amp;$W50&amp;$X50&amp;$Y50&amp;$Z50&amp;$AA50&amp;$AB50&amp;$AC50&amp;$AD50&amp;$AE50&amp;$AF50&amp;$AG50&amp;$AH50&amp;$AI50&amp;$AJ50))</x:f>
+      </x:c>
+      <x:c r="M50" s="341"/>
       <x:c r="N50"/>
       <x:c r="O50"/>
       <x:c r="P50"/>
@@ -7609,33 +7897,35 @@
       </x:c>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
-      <x:c r="A51" s="294"/>
-      <x:c r="B51" s="294"/>
-      <x:c r="C51" s="294"/>
-      <x:c r="D51" s="294" t="str">
+      <x:c r="A51" s="346"/>
+      <x:c r="B51" s="346"/>
+      <x:c r="C51" s="346"/>
+      <x:c r="D51" s="346" t="str">
         <x:f>IF($A51="Verdadero o Falso Simple","Verdadero",IF($A51="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A51="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E51" s="294" t="str">
+      <x:c r="E51" s="346" t="str">
         <x:f>IF($A51="Verdadero o Falso Simple","Falso",IF($A51="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A51="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F51" s="294" t="str">
+      <x:c r="F51" s="346" t="str">
         <x:f>IF($A51="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A51="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G51" s="294" t="str">
+      <x:c r="G51" s="346" t="str">
         <x:f>IF($A51="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A51="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H51" s="294" t="str">
+      <x:c r="H51" s="346" t="str">
         <x:f>IF($A51="Verdadero o Falso Simple","",IF($A51="Respuesta A/B/Ambas/Ninguna","",IF($A51="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I51" s="294"/>
-      <x:c r="J51" s="294" t="n">
+      <x:c r="I51" s="346"/>
+      <x:c r="J51" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K51" s="294" t="str">
+      <x:c r="K51" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L51" s="295"/>
-      <x:c r="M51" s="289"/>
+      <x:c r="L51" s="347" t="str">
+        <x:f>IF(TRIM($A51)="","",IF(COUNTIF($Q51:$AJ51,"?*")=0,"OK","Falta revisar: "&amp;$Q51&amp;$R51&amp;$S51&amp;$T51&amp;$U51&amp;$V51&amp;$W51&amp;$X51&amp;$Y51&amp;$Z51&amp;$AA51&amp;$AB51&amp;$AC51&amp;$AD51&amp;$AE51&amp;$AF51&amp;$AG51&amp;$AH51&amp;$AI51&amp;$AJ51))</x:f>
+      </x:c>
+      <x:c r="M51" s="341"/>
       <x:c r="N51"/>
       <x:c r="O51"/>
       <x:c r="P51"/>
@@ -7714,33 +8004,35 @@
       </x:c>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
-      <x:c r="A52" s="294"/>
-      <x:c r="B52" s="294"/>
-      <x:c r="C52" s="294"/>
-      <x:c r="D52" s="294" t="str">
+      <x:c r="A52" s="346"/>
+      <x:c r="B52" s="346"/>
+      <x:c r="C52" s="346"/>
+      <x:c r="D52" s="346" t="str">
         <x:f>IF($A52="Verdadero o Falso Simple","Verdadero",IF($A52="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A52="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E52" s="294" t="str">
+      <x:c r="E52" s="346" t="str">
         <x:f>IF($A52="Verdadero o Falso Simple","Falso",IF($A52="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A52="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F52" s="294" t="str">
+      <x:c r="F52" s="346" t="str">
         <x:f>IF($A52="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A52="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G52" s="294" t="str">
+      <x:c r="G52" s="346" t="str">
         <x:f>IF($A52="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A52="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H52" s="294" t="str">
+      <x:c r="H52" s="346" t="str">
         <x:f>IF($A52="Verdadero o Falso Simple","",IF($A52="Respuesta A/B/Ambas/Ninguna","",IF($A52="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I52" s="294"/>
-      <x:c r="J52" s="294" t="n">
+      <x:c r="I52" s="346"/>
+      <x:c r="J52" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K52" s="294" t="str">
+      <x:c r="K52" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L52" s="295"/>
-      <x:c r="M52" s="289"/>
+      <x:c r="L52" s="347" t="str">
+        <x:f>IF(TRIM($A52)="","",IF(COUNTIF($Q52:$AJ52,"?*")=0,"OK","Falta revisar: "&amp;$Q52&amp;$R52&amp;$S52&amp;$T52&amp;$U52&amp;$V52&amp;$W52&amp;$X52&amp;$Y52&amp;$Z52&amp;$AA52&amp;$AB52&amp;$AC52&amp;$AD52&amp;$AE52&amp;$AF52&amp;$AG52&amp;$AH52&amp;$AI52&amp;$AJ52))</x:f>
+      </x:c>
+      <x:c r="M52" s="341"/>
       <x:c r="N52"/>
       <x:c r="O52"/>
       <x:c r="P52"/>
@@ -7819,33 +8111,35 @@
       </x:c>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
-      <x:c r="A53" s="294"/>
-      <x:c r="B53" s="294"/>
-      <x:c r="C53" s="294"/>
-      <x:c r="D53" s="294" t="str">
+      <x:c r="A53" s="346"/>
+      <x:c r="B53" s="346"/>
+      <x:c r="C53" s="346"/>
+      <x:c r="D53" s="346" t="str">
         <x:f>IF($A53="Verdadero o Falso Simple","Verdadero",IF($A53="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A53="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E53" s="294" t="str">
+      <x:c r="E53" s="346" t="str">
         <x:f>IF($A53="Verdadero o Falso Simple","Falso",IF($A53="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A53="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F53" s="294" t="str">
+      <x:c r="F53" s="346" t="str">
         <x:f>IF($A53="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A53="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G53" s="294" t="str">
+      <x:c r="G53" s="346" t="str">
         <x:f>IF($A53="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A53="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H53" s="294" t="str">
+      <x:c r="H53" s="346" t="str">
         <x:f>IF($A53="Verdadero o Falso Simple","",IF($A53="Respuesta A/B/Ambas/Ninguna","",IF($A53="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I53" s="294"/>
-      <x:c r="J53" s="294" t="n">
+      <x:c r="I53" s="346"/>
+      <x:c r="J53" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K53" s="294" t="str">
+      <x:c r="K53" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L53" s="295"/>
-      <x:c r="M53" s="289"/>
+      <x:c r="L53" s="347" t="str">
+        <x:f>IF(TRIM($A53)="","",IF(COUNTIF($Q53:$AJ53,"?*")=0,"OK","Falta revisar: "&amp;$Q53&amp;$R53&amp;$S53&amp;$T53&amp;$U53&amp;$V53&amp;$W53&amp;$X53&amp;$Y53&amp;$Z53&amp;$AA53&amp;$AB53&amp;$AC53&amp;$AD53&amp;$AE53&amp;$AF53&amp;$AG53&amp;$AH53&amp;$AI53&amp;$AJ53))</x:f>
+      </x:c>
+      <x:c r="M53" s="341"/>
       <x:c r="N53"/>
       <x:c r="O53"/>
       <x:c r="P53"/>
@@ -7924,33 +8218,35 @@
       </x:c>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
-      <x:c r="A54" s="294"/>
-      <x:c r="B54" s="294"/>
-      <x:c r="C54" s="294"/>
-      <x:c r="D54" s="294" t="str">
+      <x:c r="A54" s="346"/>
+      <x:c r="B54" s="346"/>
+      <x:c r="C54" s="346"/>
+      <x:c r="D54" s="346" t="str">
         <x:f>IF($A54="Verdadero o Falso Simple","Verdadero",IF($A54="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A54="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E54" s="294" t="str">
+      <x:c r="E54" s="346" t="str">
         <x:f>IF($A54="Verdadero o Falso Simple","Falso",IF($A54="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A54="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F54" s="294" t="str">
+      <x:c r="F54" s="346" t="str">
         <x:f>IF($A54="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A54="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G54" s="294" t="str">
+      <x:c r="G54" s="346" t="str">
         <x:f>IF($A54="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A54="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H54" s="294" t="str">
+      <x:c r="H54" s="346" t="str">
         <x:f>IF($A54="Verdadero o Falso Simple","",IF($A54="Respuesta A/B/Ambas/Ninguna","",IF($A54="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I54" s="294"/>
-      <x:c r="J54" s="294" t="n">
+      <x:c r="I54" s="346"/>
+      <x:c r="J54" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K54" s="294" t="str">
+      <x:c r="K54" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L54" s="295"/>
-      <x:c r="M54" s="289"/>
+      <x:c r="L54" s="347" t="str">
+        <x:f>IF(TRIM($A54)="","",IF(COUNTIF($Q54:$AJ54,"?*")=0,"OK","Falta revisar: "&amp;$Q54&amp;$R54&amp;$S54&amp;$T54&amp;$U54&amp;$V54&amp;$W54&amp;$X54&amp;$Y54&amp;$Z54&amp;$AA54&amp;$AB54&amp;$AC54&amp;$AD54&amp;$AE54&amp;$AF54&amp;$AG54&amp;$AH54&amp;$AI54&amp;$AJ54))</x:f>
+      </x:c>
+      <x:c r="M54" s="341"/>
       <x:c r="N54"/>
       <x:c r="O54"/>
       <x:c r="P54"/>
@@ -8029,33 +8325,35 @@
       </x:c>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
-      <x:c r="A55" s="294"/>
-      <x:c r="B55" s="294"/>
-      <x:c r="C55" s="294"/>
-      <x:c r="D55" s="294" t="str">
+      <x:c r="A55" s="346"/>
+      <x:c r="B55" s="346"/>
+      <x:c r="C55" s="346"/>
+      <x:c r="D55" s="346" t="str">
         <x:f>IF($A55="Verdadero o Falso Simple","Verdadero",IF($A55="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A55="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E55" s="294" t="str">
+      <x:c r="E55" s="346" t="str">
         <x:f>IF($A55="Verdadero o Falso Simple","Falso",IF($A55="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A55="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F55" s="294" t="str">
+      <x:c r="F55" s="346" t="str">
         <x:f>IF($A55="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A55="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G55" s="294" t="str">
+      <x:c r="G55" s="346" t="str">
         <x:f>IF($A55="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A55="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H55" s="294" t="str">
+      <x:c r="H55" s="346" t="str">
         <x:f>IF($A55="Verdadero o Falso Simple","",IF($A55="Respuesta A/B/Ambas/Ninguna","",IF($A55="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I55" s="294"/>
-      <x:c r="J55" s="294" t="n">
+      <x:c r="I55" s="346"/>
+      <x:c r="J55" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K55" s="294" t="str">
+      <x:c r="K55" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L55" s="295"/>
-      <x:c r="M55" s="289"/>
+      <x:c r="L55" s="347" t="str">
+        <x:f>IF(TRIM($A55)="","",IF(COUNTIF($Q55:$AJ55,"?*")=0,"OK","Falta revisar: "&amp;$Q55&amp;$R55&amp;$S55&amp;$T55&amp;$U55&amp;$V55&amp;$W55&amp;$X55&amp;$Y55&amp;$Z55&amp;$AA55&amp;$AB55&amp;$AC55&amp;$AD55&amp;$AE55&amp;$AF55&amp;$AG55&amp;$AH55&amp;$AI55&amp;$AJ55))</x:f>
+      </x:c>
+      <x:c r="M55" s="341"/>
       <x:c r="N55"/>
       <x:c r="O55"/>
       <x:c r="P55"/>
@@ -8134,33 +8432,35 @@
       </x:c>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
-      <x:c r="A56" s="294"/>
-      <x:c r="B56" s="294"/>
-      <x:c r="C56" s="294"/>
-      <x:c r="D56" s="294" t="str">
+      <x:c r="A56" s="346"/>
+      <x:c r="B56" s="346"/>
+      <x:c r="C56" s="346"/>
+      <x:c r="D56" s="346" t="str">
         <x:f>IF($A56="Verdadero o Falso Simple","Verdadero",IF($A56="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A56="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E56" s="294" t="str">
+      <x:c r="E56" s="346" t="str">
         <x:f>IF($A56="Verdadero o Falso Simple","Falso",IF($A56="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A56="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F56" s="294" t="str">
+      <x:c r="F56" s="346" t="str">
         <x:f>IF($A56="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A56="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G56" s="294" t="str">
+      <x:c r="G56" s="346" t="str">
         <x:f>IF($A56="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A56="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H56" s="294" t="str">
+      <x:c r="H56" s="346" t="str">
         <x:f>IF($A56="Verdadero o Falso Simple","",IF($A56="Respuesta A/B/Ambas/Ninguna","",IF($A56="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I56" s="294"/>
-      <x:c r="J56" s="294" t="n">
+      <x:c r="I56" s="346"/>
+      <x:c r="J56" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K56" s="294" t="str">
+      <x:c r="K56" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L56" s="295"/>
-      <x:c r="M56" s="289"/>
+      <x:c r="L56" s="347" t="str">
+        <x:f>IF(TRIM($A56)="","",IF(COUNTIF($Q56:$AJ56,"?*")=0,"OK","Falta revisar: "&amp;$Q56&amp;$R56&amp;$S56&amp;$T56&amp;$U56&amp;$V56&amp;$W56&amp;$X56&amp;$Y56&amp;$Z56&amp;$AA56&amp;$AB56&amp;$AC56&amp;$AD56&amp;$AE56&amp;$AF56&amp;$AG56&amp;$AH56&amp;$AI56&amp;$AJ56))</x:f>
+      </x:c>
+      <x:c r="M56" s="341"/>
       <x:c r="N56"/>
       <x:c r="O56"/>
       <x:c r="P56"/>
@@ -8239,33 +8539,35 @@
       </x:c>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
-      <x:c r="A57" s="294"/>
-      <x:c r="B57" s="294"/>
-      <x:c r="C57" s="294"/>
-      <x:c r="D57" s="294" t="str">
+      <x:c r="A57" s="346"/>
+      <x:c r="B57" s="346"/>
+      <x:c r="C57" s="346"/>
+      <x:c r="D57" s="346" t="str">
         <x:f>IF($A57="Verdadero o Falso Simple","Verdadero",IF($A57="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A57="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E57" s="294" t="str">
+      <x:c r="E57" s="346" t="str">
         <x:f>IF($A57="Verdadero o Falso Simple","Falso",IF($A57="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A57="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F57" s="294" t="str">
+      <x:c r="F57" s="346" t="str">
         <x:f>IF($A57="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A57="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G57" s="294" t="str">
+      <x:c r="G57" s="346" t="str">
         <x:f>IF($A57="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A57="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H57" s="294" t="str">
+      <x:c r="H57" s="346" t="str">
         <x:f>IF($A57="Verdadero o Falso Simple","",IF($A57="Respuesta A/B/Ambas/Ninguna","",IF($A57="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I57" s="294"/>
-      <x:c r="J57" s="294" t="n">
+      <x:c r="I57" s="346"/>
+      <x:c r="J57" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K57" s="294" t="str">
+      <x:c r="K57" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L57" s="295"/>
-      <x:c r="M57" s="289"/>
+      <x:c r="L57" s="347" t="str">
+        <x:f>IF(TRIM($A57)="","",IF(COUNTIF($Q57:$AJ57,"?*")=0,"OK","Falta revisar: "&amp;$Q57&amp;$R57&amp;$S57&amp;$T57&amp;$U57&amp;$V57&amp;$W57&amp;$X57&amp;$Y57&amp;$Z57&amp;$AA57&amp;$AB57&amp;$AC57&amp;$AD57&amp;$AE57&amp;$AF57&amp;$AG57&amp;$AH57&amp;$AI57&amp;$AJ57))</x:f>
+      </x:c>
+      <x:c r="M57" s="341"/>
       <x:c r="N57"/>
       <x:c r="O57"/>
       <x:c r="P57"/>
@@ -8344,33 +8646,35 @@
       </x:c>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
-      <x:c r="A58" s="294"/>
-      <x:c r="B58" s="294"/>
-      <x:c r="C58" s="294"/>
-      <x:c r="D58" s="294" t="str">
+      <x:c r="A58" s="346"/>
+      <x:c r="B58" s="346"/>
+      <x:c r="C58" s="346"/>
+      <x:c r="D58" s="346" t="str">
         <x:f>IF($A58="Verdadero o Falso Simple","Verdadero",IF($A58="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A58="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E58" s="294" t="str">
+      <x:c r="E58" s="346" t="str">
         <x:f>IF($A58="Verdadero o Falso Simple","Falso",IF($A58="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A58="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F58" s="294" t="str">
+      <x:c r="F58" s="346" t="str">
         <x:f>IF($A58="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A58="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G58" s="294" t="str">
+      <x:c r="G58" s="346" t="str">
         <x:f>IF($A58="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A58="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H58" s="294" t="str">
+      <x:c r="H58" s="346" t="str">
         <x:f>IF($A58="Verdadero o Falso Simple","",IF($A58="Respuesta A/B/Ambas/Ninguna","",IF($A58="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I58" s="294"/>
-      <x:c r="J58" s="294" t="n">
+      <x:c r="I58" s="346"/>
+      <x:c r="J58" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K58" s="294" t="str">
+      <x:c r="K58" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L58" s="295"/>
-      <x:c r="M58" s="289"/>
+      <x:c r="L58" s="347" t="str">
+        <x:f>IF(TRIM($A58)="","",IF(COUNTIF($Q58:$AJ58,"?*")=0,"OK","Falta revisar: "&amp;$Q58&amp;$R58&amp;$S58&amp;$T58&amp;$U58&amp;$V58&amp;$W58&amp;$X58&amp;$Y58&amp;$Z58&amp;$AA58&amp;$AB58&amp;$AC58&amp;$AD58&amp;$AE58&amp;$AF58&amp;$AG58&amp;$AH58&amp;$AI58&amp;$AJ58))</x:f>
+      </x:c>
+      <x:c r="M58" s="341"/>
       <x:c r="N58"/>
       <x:c r="O58"/>
       <x:c r="P58"/>
@@ -8449,33 +8753,35 @@
       </x:c>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
-      <x:c r="A59" s="294"/>
-      <x:c r="B59" s="294"/>
-      <x:c r="C59" s="294"/>
-      <x:c r="D59" s="294" t="str">
+      <x:c r="A59" s="346"/>
+      <x:c r="B59" s="346"/>
+      <x:c r="C59" s="346"/>
+      <x:c r="D59" s="346" t="str">
         <x:f>IF($A59="Verdadero o Falso Simple","Verdadero",IF($A59="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A59="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E59" s="294" t="str">
+      <x:c r="E59" s="346" t="str">
         <x:f>IF($A59="Verdadero o Falso Simple","Falso",IF($A59="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A59="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F59" s="294" t="str">
+      <x:c r="F59" s="346" t="str">
         <x:f>IF($A59="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A59="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G59" s="294" t="str">
+      <x:c r="G59" s="346" t="str">
         <x:f>IF($A59="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A59="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H59" s="294" t="str">
+      <x:c r="H59" s="346" t="str">
         <x:f>IF($A59="Verdadero o Falso Simple","",IF($A59="Respuesta A/B/Ambas/Ninguna","",IF($A59="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I59" s="294"/>
-      <x:c r="J59" s="294" t="n">
+      <x:c r="I59" s="346"/>
+      <x:c r="J59" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K59" s="294" t="str">
+      <x:c r="K59" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L59" s="295"/>
-      <x:c r="M59" s="289"/>
+      <x:c r="L59" s="347" t="str">
+        <x:f>IF(TRIM($A59)="","",IF(COUNTIF($Q59:$AJ59,"?*")=0,"OK","Falta revisar: "&amp;$Q59&amp;$R59&amp;$S59&amp;$T59&amp;$U59&amp;$V59&amp;$W59&amp;$X59&amp;$Y59&amp;$Z59&amp;$AA59&amp;$AB59&amp;$AC59&amp;$AD59&amp;$AE59&amp;$AF59&amp;$AG59&amp;$AH59&amp;$AI59&amp;$AJ59))</x:f>
+      </x:c>
+      <x:c r="M59" s="341"/>
       <x:c r="N59"/>
       <x:c r="O59"/>
       <x:c r="P59"/>
@@ -8554,33 +8860,35 @@
       </x:c>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
-      <x:c r="A60" s="294"/>
-      <x:c r="B60" s="294"/>
-      <x:c r="C60" s="294"/>
-      <x:c r="D60" s="294" t="str">
+      <x:c r="A60" s="346"/>
+      <x:c r="B60" s="346"/>
+      <x:c r="C60" s="346"/>
+      <x:c r="D60" s="346" t="str">
         <x:f>IF($A60="Verdadero o Falso Simple","Verdadero",IF($A60="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A60="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E60" s="294" t="str">
+      <x:c r="E60" s="346" t="str">
         <x:f>IF($A60="Verdadero o Falso Simple","Falso",IF($A60="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A60="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F60" s="294" t="str">
+      <x:c r="F60" s="346" t="str">
         <x:f>IF($A60="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A60="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G60" s="294" t="str">
+      <x:c r="G60" s="346" t="str">
         <x:f>IF($A60="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A60="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H60" s="294" t="str">
+      <x:c r="H60" s="346" t="str">
         <x:f>IF($A60="Verdadero o Falso Simple","",IF($A60="Respuesta A/B/Ambas/Ninguna","",IF($A60="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I60" s="294"/>
-      <x:c r="J60" s="294" t="n">
+      <x:c r="I60" s="346"/>
+      <x:c r="J60" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K60" s="294" t="str">
+      <x:c r="K60" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L60" s="295"/>
-      <x:c r="M60" s="289"/>
+      <x:c r="L60" s="347" t="str">
+        <x:f>IF(TRIM($A60)="","",IF(COUNTIF($Q60:$AJ60,"?*")=0,"OK","Falta revisar: "&amp;$Q60&amp;$R60&amp;$S60&amp;$T60&amp;$U60&amp;$V60&amp;$W60&amp;$X60&amp;$Y60&amp;$Z60&amp;$AA60&amp;$AB60&amp;$AC60&amp;$AD60&amp;$AE60&amp;$AF60&amp;$AG60&amp;$AH60&amp;$AI60&amp;$AJ60))</x:f>
+      </x:c>
+      <x:c r="M60" s="341"/>
       <x:c r="N60"/>
       <x:c r="O60"/>
       <x:c r="P60"/>
@@ -8659,33 +8967,35 @@
       </x:c>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
-      <x:c r="A61" s="294"/>
-      <x:c r="B61" s="294"/>
-      <x:c r="C61" s="294"/>
-      <x:c r="D61" s="294" t="str">
+      <x:c r="A61" s="346"/>
+      <x:c r="B61" s="346"/>
+      <x:c r="C61" s="346"/>
+      <x:c r="D61" s="346" t="str">
         <x:f>IF($A61="Verdadero o Falso Simple","Verdadero",IF($A61="Respuesta A/B/Ambas/Ninguna","A. Si la primera es verdadera",IF($A61="Verdadero o Falso Complejas","1. ","")))</x:f>
       </x:c>
-      <x:c r="E61" s="294" t="str">
+      <x:c r="E61" s="346" t="str">
         <x:f>IF($A61="Verdadero o Falso Simple","Falso",IF($A61="Respuesta A/B/Ambas/Ninguna","B. Si la segunda es verdadera",IF($A61="Verdadero o Falso Complejas","2. ","")))</x:f>
       </x:c>
-      <x:c r="F61" s="294" t="str">
+      <x:c r="F61" s="346" t="str">
         <x:f>IF($A61="Respuesta A/B/Ambas/Ninguna","C. Si ambas son verdaderas",IF($A61="Verdadero o Falso Complejas","3. ",""))</x:f>
       </x:c>
-      <x:c r="G61" s="294" t="str">
+      <x:c r="G61" s="346" t="str">
         <x:f>IF($A61="Respuesta A/B/Ambas/Ninguna","D. Si ninguna es verdadera",IF($A61="Verdadero o Falso Complejas","4. ",""))</x:f>
       </x:c>
-      <x:c r="H61" s="294" t="str">
+      <x:c r="H61" s="346" t="str">
         <x:f>IF($A61="Verdadero o Falso Simple","",IF($A61="Respuesta A/B/Ambas/Ninguna","",IF($A61="Verdadero o Falso Complejas","","")))</x:f>
       </x:c>
-      <x:c r="I61" s="294"/>
-      <x:c r="J61" s="294" t="n">
+      <x:c r="I61" s="346"/>
+      <x:c r="J61" s="346" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K61" s="294" t="str">
+      <x:c r="K61" s="346" t="str">
         <x:v>1P</x:v>
       </x:c>
-      <x:c r="L61" s="295"/>
-      <x:c r="M61" s="289"/>
+      <x:c r="L61" s="347" t="str">
+        <x:f>IF(TRIM($A61)="","",IF(COUNTIF($Q61:$AJ61,"?*")=0,"OK","Falta revisar: "&amp;$Q61&amp;$R61&amp;$S61&amp;$T61&amp;$U61&amp;$V61&amp;$W61&amp;$X61&amp;$Y61&amp;$Z61&amp;$AA61&amp;$AB61&amp;$AC61&amp;$AD61&amp;$AE61&amp;$AF61&amp;$AG61&amp;$AH61&amp;$AI61&amp;$AJ61))</x:f>
+      </x:c>
+      <x:c r="M61" s="341"/>
       <x:c r="N61"/>
       <x:c r="O61"/>
       <x:c r="P61"/>
@@ -13319,7 +13629,7 @@
     <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Dificultad invalida" error="Use 1, 2 o 3. Casos/problemas y Emparejamiento Ampliado no llevan dificultad." sqref="J9">
       <x:formula1>INDIRECT(IF(ISNUMBER(MATCH($A9,TIPOS_SIN_DIFICULTAD,0)),"RESP_VACIA","DIFICULTADES_123"))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Tipo de pregunta" prompt="Seleccione un tipo. Las columnas de incisos se completan automÃ¡ticamente segÃºn la tipologÃ­a." errorTitle="Tipo no vÃ¡lido" error="Seleccione un tipo desde la lista del formato oficial." sqref="A2:A61">
+    <x:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Tipo de pregunta" prompt="Seleccione un tipo. Las columnas de incisos se completan automáticamente según la tipología." errorTitle="Tipo no válido" error="Seleccione un tipo desde la lista del formato oficial." sqref="A2:A61">
       <x:formula1>LISTA_TIPOS_2P</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>